<commit_message>
Update data - Thu Oct 22 08:11:48 EET 2026
</commit_message>
<xml_diff>
--- a/DEVELOPMENT_ALL_OLD_NEW/ABERCROMBIE/AB.00044 AD518.xlsx
+++ b/DEVELOPMENT_ALL_OLD_NEW/ABERCROMBIE/AB.00044 AD518.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr codeName="ThisWorkbook" hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ismailerer/Desktop/TC.DEVELOPMENT.BRAND FILE 2/ABERCROMBIE/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\TC.DEVELOPMENT.BRAND FILE 2\ABERCROMBIE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8FB5B22-AE3A-C846-AF52-19777E0ED2C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CE07EEB-1C11-4121-B9F4-E54759F0924A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="460" yWindow="1820" windowWidth="28780" windowHeight="16360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AB.0044" sheetId="29" r:id="rId1"/>
@@ -655,7 +655,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="82">
+  <borders count="83">
     <border>
       <left/>
       <right/>
@@ -717,19 +717,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color auto="1"/>
       </left>
@@ -1244,17 +1231,6 @@
         <color auto="1"/>
       </top>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -1561,19 +1537,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color indexed="8"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color indexed="8"/>
       </left>
@@ -1633,11 +1596,102 @@
     </border>
     <border>
       <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="8"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
         <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
       </left>
       <right/>
       <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
         <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="8"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
       </top>
       <bottom style="thin">
         <color indexed="64"/>
@@ -1650,56 +1704,15 @@
         <color indexed="64"/>
       </right>
       <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
         <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="8"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="18">
+  <cellStyleXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
@@ -1718,8 +1731,9 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="238">
+  <cellXfs count="250">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2"/>
@@ -1735,363 +1749,363 @@
     <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="5" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="18" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="17" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="17" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="17" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="16" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="16" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="30" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="29" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="8" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="9" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="30" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="29" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="21" fillId="2" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="23" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="20" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="25" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="19" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="5" borderId="36" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="30" fillId="0" borderId="39" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="22" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="19" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="24" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="18" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="32" fillId="5" borderId="35" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="38" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="39" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="26" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="19" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="40" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="27" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="20" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="3" borderId="40" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="40" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="40" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="41" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="3" borderId="40" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="3" borderId="40" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="3" borderId="41" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="41" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="41" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="22" fillId="5" borderId="40" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="5" borderId="40" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="3" borderId="41" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="23" fillId="3" borderId="41" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="40" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="6" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="3" borderId="42" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="5" borderId="41" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="5" borderId="41" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="38" fillId="6" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="41" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="6" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="39" fillId="6" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="40" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="5" borderId="13" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="13" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="13" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="44" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="44" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="44" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="40" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="40" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="6" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="35" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="35" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="6" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="41" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="5" borderId="14" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="14" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="14" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="45" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="45" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="45" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="26" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="40" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="40" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="35" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="51" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="52" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="53" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="53" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="36" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="36" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="53" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="53" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="36" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="53" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="54" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="55" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="55" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="53" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="56" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="6" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="65" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="55" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="55" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="65" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="6" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="55" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="58" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="6" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="59" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="60" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="40" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="6" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="61" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="62" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="41" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="41" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="43" fillId="4" borderId="50" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="40" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="43" fillId="4" borderId="48" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="28" fillId="4" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="43" fillId="4" borderId="28" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="43" fillId="4" borderId="27" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="28" fillId="4" borderId="13" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="28" fillId="4" borderId="12" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="16" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="68" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="15" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="66" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="69" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="16" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="67" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="15" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="68" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="67" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="67" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="66" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="70" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="69" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="69" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="18" fillId="3" borderId="67" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="3" borderId="67" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="68" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="73" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="3" borderId="69" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="3" borderId="69" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="67" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="69" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="71" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="31" fillId="4" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="31" fillId="4" borderId="66" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="31" fillId="4" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="4" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="31" fillId="3" borderId="67" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="27" fillId="3" borderId="47" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="27" fillId="3" borderId="61" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="27" fillId="3" borderId="21" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="47" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="61" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="3" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="3" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="3" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="69" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="71" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="74" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="31" fillId="4" borderId="16" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="31" fillId="4" borderId="68" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="31" fillId="4" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="4" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="31" fillId="3" borderId="69" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="27" fillId="3" borderId="49" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="27" fillId="3" borderId="63" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="27" fillId="3" borderId="22" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="49" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="63" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="3" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="3" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="53" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="3" borderId="53" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="3" borderId="53" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="3" borderId="53" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="3" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="41" fillId="3" borderId="54" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="3" borderId="61" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="67" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="67" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="67" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="69" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="55" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="3" borderId="55" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="3" borderId="55" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="3" borderId="55" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="3" borderId="56" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="3" borderId="63" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="69" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="69" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="69" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="41" fillId="0" borderId="71" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="74" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="31" fillId="4" borderId="41" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="31" fillId="4" borderId="40" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="45" fillId="4" borderId="75" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="45" fillId="4" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="41" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="42" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="42" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="3" borderId="76" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="31" fillId="3" borderId="76" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="3" borderId="76" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="40" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="41" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="41" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="3" borderId="73" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="31" fillId="3" borderId="73" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="3" borderId="73" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="18" fillId="3" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2103,352 +2117,388 @@
     <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="79" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="57" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="80" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="46" fillId="5" borderId="75" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="74" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="55" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="75" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="5" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="29" fillId="3" borderId="80" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="28" fillId="3" borderId="79" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="29" fillId="3" borderId="75" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="28" fillId="3" borderId="74" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="28" fillId="3" borderId="66" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="28" fillId="3" borderId="64" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="28" fillId="3" borderId="57" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="28" fillId="3" borderId="55" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="3" borderId="80" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="17" fillId="3" borderId="75" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="80" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="5" borderId="80" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="80" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="75" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="5" borderId="75" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="75" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="80" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="75" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="80" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="40" fillId="0" borderId="80" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="40" fillId="0" borderId="80" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="75" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="40" fillId="0" borderId="75" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="40" fillId="0" borderId="75" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="3" borderId="80" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="23" fillId="3" borderId="80" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="23" fillId="3" borderId="75" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="3" borderId="75" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="3" borderId="80" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="3" borderId="79" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="3" borderId="57" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="6" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="6" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="41" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="41" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="80" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="55" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="69" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="72" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="71" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="74" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="59" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="60" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="61" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="62" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="53" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="54" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="28" fillId="4" borderId="43" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="26" fillId="3" borderId="75" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="3" borderId="74" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="3" borderId="55" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="5" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="5" borderId="20" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="14" fontId="28" fillId="4" borderId="66" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="23" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="14" fontId="28" fillId="4" borderId="65" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="21" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="14" fontId="31" fillId="4" borderId="21" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="14" fontId="22" fillId="0" borderId="20" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="14" fontId="31" fillId="4" borderId="24" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="14" fontId="22" fillId="0" borderId="23" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="31" fillId="4" borderId="31" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="31" fillId="4" borderId="32" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="31" fillId="4" borderId="33" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="2" borderId="7" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="2" borderId="8" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="2" borderId="11" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="2" borderId="12" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="2" borderId="34" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="2" borderId="35" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="43" fillId="4" borderId="81" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="43" fillId="4" borderId="66" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="43" fillId="4" borderId="57" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="4" borderId="79" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="4" borderId="66" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="4" borderId="57" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="43" fillId="4" borderId="79" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="28" fillId="4" borderId="57" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="21" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="24" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="22" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="22" fillId="0" borderId="21" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="22" fillId="0" borderId="24" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="22" fillId="0" borderId="22" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="28" fillId="4" borderId="51" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="28" fillId="4" borderId="52" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="22" fillId="0" borderId="21" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="14" fontId="22" fillId="0" borderId="24" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="14" fontId="31" fillId="4" borderId="36" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="22" fillId="0" borderId="22" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="44" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="46" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="3" borderId="49" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="3" borderId="22" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="41" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="4" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="36" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="56" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="57" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="15" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="17" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="27" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="12" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="41" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="31" fillId="4" borderId="21" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="31" fillId="4" borderId="48" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="31" fillId="4" borderId="6" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="16" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="29" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="5" borderId="21" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="24" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="22" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="14" fontId="31" fillId="4" borderId="37" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="14" fontId="31" fillId="4" borderId="38" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="31" fillId="4" borderId="35" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="31" fillId="4" borderId="46" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="59" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="60" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="14" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="16" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="51" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="52" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="26" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="11" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="40" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="31" fillId="4" borderId="36" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="31" fillId="4" borderId="47" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="15" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="28" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="43" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="45" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="40" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="6" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="6" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="54" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="41" fillId="0" borderId="55" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="77" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="28" fillId="4" borderId="42" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="28" fillId="4" borderId="64" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="28" fillId="4" borderId="63" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="31" fillId="4" borderId="20" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="31" fillId="4" borderId="23" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="31" fillId="4" borderId="30" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="31" fillId="4" borderId="31" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="31" fillId="4" borderId="32" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="2" borderId="6" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="2" borderId="7" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="2" borderId="10" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="2" borderId="11" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="2" borderId="33" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="2" borderId="34" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="43" fillId="4" borderId="76" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="43" fillId="4" borderId="64" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="43" fillId="4" borderId="55" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="74" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="64" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="55" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="43" fillId="4" borderId="74" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="28" fillId="4" borderId="55" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="20" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="23" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="21" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="22" fillId="0" borderId="20" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="22" fillId="0" borderId="23" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="22" fillId="0" borderId="21" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="28" fillId="4" borderId="49" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="28" fillId="4" borderId="50" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="57" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="58" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="6" borderId="79" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="6" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="79" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="78" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="79" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="78" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="5" borderId="79" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="5" borderId="78" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="31" fillId="4" borderId="79" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="31" fillId="4" borderId="77" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="31" fillId="4" borderId="78" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="79" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="78" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="79" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="78" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="79" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="78" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="3" borderId="79" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="3" borderId="78" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="79" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="78" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="79" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="81" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="81" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="79" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="78" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="79" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="3" borderId="78" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="5" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="82" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="82" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="82" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="82" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="18">
+  <cellStyles count="19">
     <cellStyle name="Currency 2" xfId="5" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
     <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="9" builtinId="9" hidden="1"/>
@@ -2466,6 +2516,7 @@
     <cellStyle name="Normal 10 10 3" xfId="1" xr:uid="{00000000-0005-0000-0000-00000E000000}"/>
     <cellStyle name="Normal 2" xfId="2" xr:uid="{00000000-0005-0000-0000-00000F000000}"/>
     <cellStyle name="Normal 3" xfId="3" xr:uid="{00000000-0005-0000-0000-000010000000}"/>
+    <cellStyle name="Normal 3 2" xfId="18" xr:uid="{C6202B95-B98A-4AC2-AD62-B6C8735224C6}"/>
     <cellStyle name="Normal_0136" xfId="4" xr:uid="{00000000-0005-0000-0000-000011000000}"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -2748,779 +2799,779 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:M92"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="13.2"/>
   <cols>
-    <col min="1" max="1" width="12.83203125" style="3" customWidth="1"/>
+    <col min="1" max="1" width="12.77734375" style="3" customWidth="1"/>
     <col min="2" max="2" width="134" style="3" customWidth="1"/>
     <col min="3" max="3" width="48" style="3" customWidth="1"/>
     <col min="4" max="4" width="46.33203125" style="3" customWidth="1"/>
     <col min="5" max="5" width="63.6640625" style="3" customWidth="1"/>
     <col min="6" max="6" width="56" style="3" customWidth="1"/>
-    <col min="7" max="7" width="47.1640625" style="3" customWidth="1"/>
+    <col min="7" max="7" width="47.109375" style="3" customWidth="1"/>
     <col min="8" max="8" width="52.33203125" style="3" customWidth="1"/>
-    <col min="9" max="9" width="106.1640625" style="3" customWidth="1"/>
-    <col min="10" max="10" width="65.1640625" style="3" customWidth="1"/>
-    <col min="11" max="11" width="28.83203125" style="3" customWidth="1"/>
-    <col min="12" max="256" width="8.83203125" style="3"/>
+    <col min="9" max="9" width="106.109375" style="3" customWidth="1"/>
+    <col min="10" max="10" width="65.109375" style="3" customWidth="1"/>
+    <col min="11" max="11" width="28.77734375" style="3" customWidth="1"/>
+    <col min="12" max="256" width="8.77734375" style="3"/>
     <col min="257" max="257" width="2.33203125" style="3" customWidth="1"/>
     <col min="258" max="258" width="57.6640625" style="3" customWidth="1"/>
     <col min="259" max="259" width="18.6640625" style="3" customWidth="1"/>
-    <col min="260" max="260" width="17.1640625" style="3" customWidth="1"/>
-    <col min="261" max="261" width="13.83203125" style="3" customWidth="1"/>
-    <col min="262" max="262" width="11.1640625" style="3" customWidth="1"/>
-    <col min="263" max="263" width="23.5" style="3" customWidth="1"/>
-    <col min="264" max="264" width="44.1640625" style="3" customWidth="1"/>
-    <col min="265" max="265" width="26.5" style="3" customWidth="1"/>
-    <col min="266" max="266" width="34.1640625" style="3" customWidth="1"/>
+    <col min="260" max="260" width="17.109375" style="3" customWidth="1"/>
+    <col min="261" max="261" width="13.77734375" style="3" customWidth="1"/>
+    <col min="262" max="262" width="11.109375" style="3" customWidth="1"/>
+    <col min="263" max="263" width="23.44140625" style="3" customWidth="1"/>
+    <col min="264" max="264" width="44.109375" style="3" customWidth="1"/>
+    <col min="265" max="265" width="26.44140625" style="3" customWidth="1"/>
+    <col min="266" max="266" width="34.109375" style="3" customWidth="1"/>
     <col min="267" max="267" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="268" max="512" width="8.83203125" style="3"/>
+    <col min="268" max="512" width="8.77734375" style="3"/>
     <col min="513" max="513" width="2.33203125" style="3" customWidth="1"/>
     <col min="514" max="514" width="57.6640625" style="3" customWidth="1"/>
     <col min="515" max="515" width="18.6640625" style="3" customWidth="1"/>
-    <col min="516" max="516" width="17.1640625" style="3" customWidth="1"/>
-    <col min="517" max="517" width="13.83203125" style="3" customWidth="1"/>
-    <col min="518" max="518" width="11.1640625" style="3" customWidth="1"/>
-    <col min="519" max="519" width="23.5" style="3" customWidth="1"/>
-    <col min="520" max="520" width="44.1640625" style="3" customWidth="1"/>
-    <col min="521" max="521" width="26.5" style="3" customWidth="1"/>
-    <col min="522" max="522" width="34.1640625" style="3" customWidth="1"/>
+    <col min="516" max="516" width="17.109375" style="3" customWidth="1"/>
+    <col min="517" max="517" width="13.77734375" style="3" customWidth="1"/>
+    <col min="518" max="518" width="11.109375" style="3" customWidth="1"/>
+    <col min="519" max="519" width="23.44140625" style="3" customWidth="1"/>
+    <col min="520" max="520" width="44.109375" style="3" customWidth="1"/>
+    <col min="521" max="521" width="26.44140625" style="3" customWidth="1"/>
+    <col min="522" max="522" width="34.109375" style="3" customWidth="1"/>
     <col min="523" max="523" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="524" max="768" width="8.83203125" style="3"/>
+    <col min="524" max="768" width="8.77734375" style="3"/>
     <col min="769" max="769" width="2.33203125" style="3" customWidth="1"/>
     <col min="770" max="770" width="57.6640625" style="3" customWidth="1"/>
     <col min="771" max="771" width="18.6640625" style="3" customWidth="1"/>
-    <col min="772" max="772" width="17.1640625" style="3" customWidth="1"/>
-    <col min="773" max="773" width="13.83203125" style="3" customWidth="1"/>
-    <col min="774" max="774" width="11.1640625" style="3" customWidth="1"/>
-    <col min="775" max="775" width="23.5" style="3" customWidth="1"/>
-    <col min="776" max="776" width="44.1640625" style="3" customWidth="1"/>
-    <col min="777" max="777" width="26.5" style="3" customWidth="1"/>
-    <col min="778" max="778" width="34.1640625" style="3" customWidth="1"/>
+    <col min="772" max="772" width="17.109375" style="3" customWidth="1"/>
+    <col min="773" max="773" width="13.77734375" style="3" customWidth="1"/>
+    <col min="774" max="774" width="11.109375" style="3" customWidth="1"/>
+    <col min="775" max="775" width="23.44140625" style="3" customWidth="1"/>
+    <col min="776" max="776" width="44.109375" style="3" customWidth="1"/>
+    <col min="777" max="777" width="26.44140625" style="3" customWidth="1"/>
+    <col min="778" max="778" width="34.109375" style="3" customWidth="1"/>
     <col min="779" max="779" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="780" max="1024" width="8.83203125" style="3"/>
+    <col min="780" max="1024" width="8.77734375" style="3"/>
     <col min="1025" max="1025" width="2.33203125" style="3" customWidth="1"/>
     <col min="1026" max="1026" width="57.6640625" style="3" customWidth="1"/>
     <col min="1027" max="1027" width="18.6640625" style="3" customWidth="1"/>
-    <col min="1028" max="1028" width="17.1640625" style="3" customWidth="1"/>
-    <col min="1029" max="1029" width="13.83203125" style="3" customWidth="1"/>
-    <col min="1030" max="1030" width="11.1640625" style="3" customWidth="1"/>
-    <col min="1031" max="1031" width="23.5" style="3" customWidth="1"/>
-    <col min="1032" max="1032" width="44.1640625" style="3" customWidth="1"/>
-    <col min="1033" max="1033" width="26.5" style="3" customWidth="1"/>
-    <col min="1034" max="1034" width="34.1640625" style="3" customWidth="1"/>
+    <col min="1028" max="1028" width="17.109375" style="3" customWidth="1"/>
+    <col min="1029" max="1029" width="13.77734375" style="3" customWidth="1"/>
+    <col min="1030" max="1030" width="11.109375" style="3" customWidth="1"/>
+    <col min="1031" max="1031" width="23.44140625" style="3" customWidth="1"/>
+    <col min="1032" max="1032" width="44.109375" style="3" customWidth="1"/>
+    <col min="1033" max="1033" width="26.44140625" style="3" customWidth="1"/>
+    <col min="1034" max="1034" width="34.109375" style="3" customWidth="1"/>
     <col min="1035" max="1035" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="1036" max="1280" width="8.83203125" style="3"/>
+    <col min="1036" max="1280" width="8.77734375" style="3"/>
     <col min="1281" max="1281" width="2.33203125" style="3" customWidth="1"/>
     <col min="1282" max="1282" width="57.6640625" style="3" customWidth="1"/>
     <col min="1283" max="1283" width="18.6640625" style="3" customWidth="1"/>
-    <col min="1284" max="1284" width="17.1640625" style="3" customWidth="1"/>
-    <col min="1285" max="1285" width="13.83203125" style="3" customWidth="1"/>
-    <col min="1286" max="1286" width="11.1640625" style="3" customWidth="1"/>
-    <col min="1287" max="1287" width="23.5" style="3" customWidth="1"/>
-    <col min="1288" max="1288" width="44.1640625" style="3" customWidth="1"/>
-    <col min="1289" max="1289" width="26.5" style="3" customWidth="1"/>
-    <col min="1290" max="1290" width="34.1640625" style="3" customWidth="1"/>
+    <col min="1284" max="1284" width="17.109375" style="3" customWidth="1"/>
+    <col min="1285" max="1285" width="13.77734375" style="3" customWidth="1"/>
+    <col min="1286" max="1286" width="11.109375" style="3" customWidth="1"/>
+    <col min="1287" max="1287" width="23.44140625" style="3" customWidth="1"/>
+    <col min="1288" max="1288" width="44.109375" style="3" customWidth="1"/>
+    <col min="1289" max="1289" width="26.44140625" style="3" customWidth="1"/>
+    <col min="1290" max="1290" width="34.109375" style="3" customWidth="1"/>
     <col min="1291" max="1291" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="1292" max="1536" width="8.83203125" style="3"/>
+    <col min="1292" max="1536" width="8.77734375" style="3"/>
     <col min="1537" max="1537" width="2.33203125" style="3" customWidth="1"/>
     <col min="1538" max="1538" width="57.6640625" style="3" customWidth="1"/>
     <col min="1539" max="1539" width="18.6640625" style="3" customWidth="1"/>
-    <col min="1540" max="1540" width="17.1640625" style="3" customWidth="1"/>
-    <col min="1541" max="1541" width="13.83203125" style="3" customWidth="1"/>
-    <col min="1542" max="1542" width="11.1640625" style="3" customWidth="1"/>
-    <col min="1543" max="1543" width="23.5" style="3" customWidth="1"/>
-    <col min="1544" max="1544" width="44.1640625" style="3" customWidth="1"/>
-    <col min="1545" max="1545" width="26.5" style="3" customWidth="1"/>
-    <col min="1546" max="1546" width="34.1640625" style="3" customWidth="1"/>
+    <col min="1540" max="1540" width="17.109375" style="3" customWidth="1"/>
+    <col min="1541" max="1541" width="13.77734375" style="3" customWidth="1"/>
+    <col min="1542" max="1542" width="11.109375" style="3" customWidth="1"/>
+    <col min="1543" max="1543" width="23.44140625" style="3" customWidth="1"/>
+    <col min="1544" max="1544" width="44.109375" style="3" customWidth="1"/>
+    <col min="1545" max="1545" width="26.44140625" style="3" customWidth="1"/>
+    <col min="1546" max="1546" width="34.109375" style="3" customWidth="1"/>
     <col min="1547" max="1547" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="1548" max="1792" width="8.83203125" style="3"/>
+    <col min="1548" max="1792" width="8.77734375" style="3"/>
     <col min="1793" max="1793" width="2.33203125" style="3" customWidth="1"/>
     <col min="1794" max="1794" width="57.6640625" style="3" customWidth="1"/>
     <col min="1795" max="1795" width="18.6640625" style="3" customWidth="1"/>
-    <col min="1796" max="1796" width="17.1640625" style="3" customWidth="1"/>
-    <col min="1797" max="1797" width="13.83203125" style="3" customWidth="1"/>
-    <col min="1798" max="1798" width="11.1640625" style="3" customWidth="1"/>
-    <col min="1799" max="1799" width="23.5" style="3" customWidth="1"/>
-    <col min="1800" max="1800" width="44.1640625" style="3" customWidth="1"/>
-    <col min="1801" max="1801" width="26.5" style="3" customWidth="1"/>
-    <col min="1802" max="1802" width="34.1640625" style="3" customWidth="1"/>
+    <col min="1796" max="1796" width="17.109375" style="3" customWidth="1"/>
+    <col min="1797" max="1797" width="13.77734375" style="3" customWidth="1"/>
+    <col min="1798" max="1798" width="11.109375" style="3" customWidth="1"/>
+    <col min="1799" max="1799" width="23.44140625" style="3" customWidth="1"/>
+    <col min="1800" max="1800" width="44.109375" style="3" customWidth="1"/>
+    <col min="1801" max="1801" width="26.44140625" style="3" customWidth="1"/>
+    <col min="1802" max="1802" width="34.109375" style="3" customWidth="1"/>
     <col min="1803" max="1803" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="1804" max="2048" width="8.83203125" style="3"/>
+    <col min="1804" max="2048" width="8.77734375" style="3"/>
     <col min="2049" max="2049" width="2.33203125" style="3" customWidth="1"/>
     <col min="2050" max="2050" width="57.6640625" style="3" customWidth="1"/>
     <col min="2051" max="2051" width="18.6640625" style="3" customWidth="1"/>
-    <col min="2052" max="2052" width="17.1640625" style="3" customWidth="1"/>
-    <col min="2053" max="2053" width="13.83203125" style="3" customWidth="1"/>
-    <col min="2054" max="2054" width="11.1640625" style="3" customWidth="1"/>
-    <col min="2055" max="2055" width="23.5" style="3" customWidth="1"/>
-    <col min="2056" max="2056" width="44.1640625" style="3" customWidth="1"/>
-    <col min="2057" max="2057" width="26.5" style="3" customWidth="1"/>
-    <col min="2058" max="2058" width="34.1640625" style="3" customWidth="1"/>
+    <col min="2052" max="2052" width="17.109375" style="3" customWidth="1"/>
+    <col min="2053" max="2053" width="13.77734375" style="3" customWidth="1"/>
+    <col min="2054" max="2054" width="11.109375" style="3" customWidth="1"/>
+    <col min="2055" max="2055" width="23.44140625" style="3" customWidth="1"/>
+    <col min="2056" max="2056" width="44.109375" style="3" customWidth="1"/>
+    <col min="2057" max="2057" width="26.44140625" style="3" customWidth="1"/>
+    <col min="2058" max="2058" width="34.109375" style="3" customWidth="1"/>
     <col min="2059" max="2059" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="2060" max="2304" width="8.83203125" style="3"/>
+    <col min="2060" max="2304" width="8.77734375" style="3"/>
     <col min="2305" max="2305" width="2.33203125" style="3" customWidth="1"/>
     <col min="2306" max="2306" width="57.6640625" style="3" customWidth="1"/>
     <col min="2307" max="2307" width="18.6640625" style="3" customWidth="1"/>
-    <col min="2308" max="2308" width="17.1640625" style="3" customWidth="1"/>
-    <col min="2309" max="2309" width="13.83203125" style="3" customWidth="1"/>
-    <col min="2310" max="2310" width="11.1640625" style="3" customWidth="1"/>
-    <col min="2311" max="2311" width="23.5" style="3" customWidth="1"/>
-    <col min="2312" max="2312" width="44.1640625" style="3" customWidth="1"/>
-    <col min="2313" max="2313" width="26.5" style="3" customWidth="1"/>
-    <col min="2314" max="2314" width="34.1640625" style="3" customWidth="1"/>
+    <col min="2308" max="2308" width="17.109375" style="3" customWidth="1"/>
+    <col min="2309" max="2309" width="13.77734375" style="3" customWidth="1"/>
+    <col min="2310" max="2310" width="11.109375" style="3" customWidth="1"/>
+    <col min="2311" max="2311" width="23.44140625" style="3" customWidth="1"/>
+    <col min="2312" max="2312" width="44.109375" style="3" customWidth="1"/>
+    <col min="2313" max="2313" width="26.44140625" style="3" customWidth="1"/>
+    <col min="2314" max="2314" width="34.109375" style="3" customWidth="1"/>
     <col min="2315" max="2315" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="2316" max="2560" width="8.83203125" style="3"/>
+    <col min="2316" max="2560" width="8.77734375" style="3"/>
     <col min="2561" max="2561" width="2.33203125" style="3" customWidth="1"/>
     <col min="2562" max="2562" width="57.6640625" style="3" customWidth="1"/>
     <col min="2563" max="2563" width="18.6640625" style="3" customWidth="1"/>
-    <col min="2564" max="2564" width="17.1640625" style="3" customWidth="1"/>
-    <col min="2565" max="2565" width="13.83203125" style="3" customWidth="1"/>
-    <col min="2566" max="2566" width="11.1640625" style="3" customWidth="1"/>
-    <col min="2567" max="2567" width="23.5" style="3" customWidth="1"/>
-    <col min="2568" max="2568" width="44.1640625" style="3" customWidth="1"/>
-    <col min="2569" max="2569" width="26.5" style="3" customWidth="1"/>
-    <col min="2570" max="2570" width="34.1640625" style="3" customWidth="1"/>
+    <col min="2564" max="2564" width="17.109375" style="3" customWidth="1"/>
+    <col min="2565" max="2565" width="13.77734375" style="3" customWidth="1"/>
+    <col min="2566" max="2566" width="11.109375" style="3" customWidth="1"/>
+    <col min="2567" max="2567" width="23.44140625" style="3" customWidth="1"/>
+    <col min="2568" max="2568" width="44.109375" style="3" customWidth="1"/>
+    <col min="2569" max="2569" width="26.44140625" style="3" customWidth="1"/>
+    <col min="2570" max="2570" width="34.109375" style="3" customWidth="1"/>
     <col min="2571" max="2571" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="2572" max="2816" width="8.83203125" style="3"/>
+    <col min="2572" max="2816" width="8.77734375" style="3"/>
     <col min="2817" max="2817" width="2.33203125" style="3" customWidth="1"/>
     <col min="2818" max="2818" width="57.6640625" style="3" customWidth="1"/>
     <col min="2819" max="2819" width="18.6640625" style="3" customWidth="1"/>
-    <col min="2820" max="2820" width="17.1640625" style="3" customWidth="1"/>
-    <col min="2821" max="2821" width="13.83203125" style="3" customWidth="1"/>
-    <col min="2822" max="2822" width="11.1640625" style="3" customWidth="1"/>
-    <col min="2823" max="2823" width="23.5" style="3" customWidth="1"/>
-    <col min="2824" max="2824" width="44.1640625" style="3" customWidth="1"/>
-    <col min="2825" max="2825" width="26.5" style="3" customWidth="1"/>
-    <col min="2826" max="2826" width="34.1640625" style="3" customWidth="1"/>
+    <col min="2820" max="2820" width="17.109375" style="3" customWidth="1"/>
+    <col min="2821" max="2821" width="13.77734375" style="3" customWidth="1"/>
+    <col min="2822" max="2822" width="11.109375" style="3" customWidth="1"/>
+    <col min="2823" max="2823" width="23.44140625" style="3" customWidth="1"/>
+    <col min="2824" max="2824" width="44.109375" style="3" customWidth="1"/>
+    <col min="2825" max="2825" width="26.44140625" style="3" customWidth="1"/>
+    <col min="2826" max="2826" width="34.109375" style="3" customWidth="1"/>
     <col min="2827" max="2827" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="2828" max="3072" width="8.83203125" style="3"/>
+    <col min="2828" max="3072" width="8.77734375" style="3"/>
     <col min="3073" max="3073" width="2.33203125" style="3" customWidth="1"/>
     <col min="3074" max="3074" width="57.6640625" style="3" customWidth="1"/>
     <col min="3075" max="3075" width="18.6640625" style="3" customWidth="1"/>
-    <col min="3076" max="3076" width="17.1640625" style="3" customWidth="1"/>
-    <col min="3077" max="3077" width="13.83203125" style="3" customWidth="1"/>
-    <col min="3078" max="3078" width="11.1640625" style="3" customWidth="1"/>
-    <col min="3079" max="3079" width="23.5" style="3" customWidth="1"/>
-    <col min="3080" max="3080" width="44.1640625" style="3" customWidth="1"/>
-    <col min="3081" max="3081" width="26.5" style="3" customWidth="1"/>
-    <col min="3082" max="3082" width="34.1640625" style="3" customWidth="1"/>
+    <col min="3076" max="3076" width="17.109375" style="3" customWidth="1"/>
+    <col min="3077" max="3077" width="13.77734375" style="3" customWidth="1"/>
+    <col min="3078" max="3078" width="11.109375" style="3" customWidth="1"/>
+    <col min="3079" max="3079" width="23.44140625" style="3" customWidth="1"/>
+    <col min="3080" max="3080" width="44.109375" style="3" customWidth="1"/>
+    <col min="3081" max="3081" width="26.44140625" style="3" customWidth="1"/>
+    <col min="3082" max="3082" width="34.109375" style="3" customWidth="1"/>
     <col min="3083" max="3083" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="3084" max="3328" width="8.83203125" style="3"/>
+    <col min="3084" max="3328" width="8.77734375" style="3"/>
     <col min="3329" max="3329" width="2.33203125" style="3" customWidth="1"/>
     <col min="3330" max="3330" width="57.6640625" style="3" customWidth="1"/>
     <col min="3331" max="3331" width="18.6640625" style="3" customWidth="1"/>
-    <col min="3332" max="3332" width="17.1640625" style="3" customWidth="1"/>
-    <col min="3333" max="3333" width="13.83203125" style="3" customWidth="1"/>
-    <col min="3334" max="3334" width="11.1640625" style="3" customWidth="1"/>
-    <col min="3335" max="3335" width="23.5" style="3" customWidth="1"/>
-    <col min="3336" max="3336" width="44.1640625" style="3" customWidth="1"/>
-    <col min="3337" max="3337" width="26.5" style="3" customWidth="1"/>
-    <col min="3338" max="3338" width="34.1640625" style="3" customWidth="1"/>
+    <col min="3332" max="3332" width="17.109375" style="3" customWidth="1"/>
+    <col min="3333" max="3333" width="13.77734375" style="3" customWidth="1"/>
+    <col min="3334" max="3334" width="11.109375" style="3" customWidth="1"/>
+    <col min="3335" max="3335" width="23.44140625" style="3" customWidth="1"/>
+    <col min="3336" max="3336" width="44.109375" style="3" customWidth="1"/>
+    <col min="3337" max="3337" width="26.44140625" style="3" customWidth="1"/>
+    <col min="3338" max="3338" width="34.109375" style="3" customWidth="1"/>
     <col min="3339" max="3339" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="3340" max="3584" width="8.83203125" style="3"/>
+    <col min="3340" max="3584" width="8.77734375" style="3"/>
     <col min="3585" max="3585" width="2.33203125" style="3" customWidth="1"/>
     <col min="3586" max="3586" width="57.6640625" style="3" customWidth="1"/>
     <col min="3587" max="3587" width="18.6640625" style="3" customWidth="1"/>
-    <col min="3588" max="3588" width="17.1640625" style="3" customWidth="1"/>
-    <col min="3589" max="3589" width="13.83203125" style="3" customWidth="1"/>
-    <col min="3590" max="3590" width="11.1640625" style="3" customWidth="1"/>
-    <col min="3591" max="3591" width="23.5" style="3" customWidth="1"/>
-    <col min="3592" max="3592" width="44.1640625" style="3" customWidth="1"/>
-    <col min="3593" max="3593" width="26.5" style="3" customWidth="1"/>
-    <col min="3594" max="3594" width="34.1640625" style="3" customWidth="1"/>
+    <col min="3588" max="3588" width="17.109375" style="3" customWidth="1"/>
+    <col min="3589" max="3589" width="13.77734375" style="3" customWidth="1"/>
+    <col min="3590" max="3590" width="11.109375" style="3" customWidth="1"/>
+    <col min="3591" max="3591" width="23.44140625" style="3" customWidth="1"/>
+    <col min="3592" max="3592" width="44.109375" style="3" customWidth="1"/>
+    <col min="3593" max="3593" width="26.44140625" style="3" customWidth="1"/>
+    <col min="3594" max="3594" width="34.109375" style="3" customWidth="1"/>
     <col min="3595" max="3595" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="3596" max="3840" width="8.83203125" style="3"/>
+    <col min="3596" max="3840" width="8.77734375" style="3"/>
     <col min="3841" max="3841" width="2.33203125" style="3" customWidth="1"/>
     <col min="3842" max="3842" width="57.6640625" style="3" customWidth="1"/>
     <col min="3843" max="3843" width="18.6640625" style="3" customWidth="1"/>
-    <col min="3844" max="3844" width="17.1640625" style="3" customWidth="1"/>
-    <col min="3845" max="3845" width="13.83203125" style="3" customWidth="1"/>
-    <col min="3846" max="3846" width="11.1640625" style="3" customWidth="1"/>
-    <col min="3847" max="3847" width="23.5" style="3" customWidth="1"/>
-    <col min="3848" max="3848" width="44.1640625" style="3" customWidth="1"/>
-    <col min="3849" max="3849" width="26.5" style="3" customWidth="1"/>
-    <col min="3850" max="3850" width="34.1640625" style="3" customWidth="1"/>
+    <col min="3844" max="3844" width="17.109375" style="3" customWidth="1"/>
+    <col min="3845" max="3845" width="13.77734375" style="3" customWidth="1"/>
+    <col min="3846" max="3846" width="11.109375" style="3" customWidth="1"/>
+    <col min="3847" max="3847" width="23.44140625" style="3" customWidth="1"/>
+    <col min="3848" max="3848" width="44.109375" style="3" customWidth="1"/>
+    <col min="3849" max="3849" width="26.44140625" style="3" customWidth="1"/>
+    <col min="3850" max="3850" width="34.109375" style="3" customWidth="1"/>
     <col min="3851" max="3851" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="3852" max="4096" width="8.83203125" style="3"/>
+    <col min="3852" max="4096" width="8.77734375" style="3"/>
     <col min="4097" max="4097" width="2.33203125" style="3" customWidth="1"/>
     <col min="4098" max="4098" width="57.6640625" style="3" customWidth="1"/>
     <col min="4099" max="4099" width="18.6640625" style="3" customWidth="1"/>
-    <col min="4100" max="4100" width="17.1640625" style="3" customWidth="1"/>
-    <col min="4101" max="4101" width="13.83203125" style="3" customWidth="1"/>
-    <col min="4102" max="4102" width="11.1640625" style="3" customWidth="1"/>
-    <col min="4103" max="4103" width="23.5" style="3" customWidth="1"/>
-    <col min="4104" max="4104" width="44.1640625" style="3" customWidth="1"/>
-    <col min="4105" max="4105" width="26.5" style="3" customWidth="1"/>
-    <col min="4106" max="4106" width="34.1640625" style="3" customWidth="1"/>
+    <col min="4100" max="4100" width="17.109375" style="3" customWidth="1"/>
+    <col min="4101" max="4101" width="13.77734375" style="3" customWidth="1"/>
+    <col min="4102" max="4102" width="11.109375" style="3" customWidth="1"/>
+    <col min="4103" max="4103" width="23.44140625" style="3" customWidth="1"/>
+    <col min="4104" max="4104" width="44.109375" style="3" customWidth="1"/>
+    <col min="4105" max="4105" width="26.44140625" style="3" customWidth="1"/>
+    <col min="4106" max="4106" width="34.109375" style="3" customWidth="1"/>
     <col min="4107" max="4107" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="4108" max="4352" width="8.83203125" style="3"/>
+    <col min="4108" max="4352" width="8.77734375" style="3"/>
     <col min="4353" max="4353" width="2.33203125" style="3" customWidth="1"/>
     <col min="4354" max="4354" width="57.6640625" style="3" customWidth="1"/>
     <col min="4355" max="4355" width="18.6640625" style="3" customWidth="1"/>
-    <col min="4356" max="4356" width="17.1640625" style="3" customWidth="1"/>
-    <col min="4357" max="4357" width="13.83203125" style="3" customWidth="1"/>
-    <col min="4358" max="4358" width="11.1640625" style="3" customWidth="1"/>
-    <col min="4359" max="4359" width="23.5" style="3" customWidth="1"/>
-    <col min="4360" max="4360" width="44.1640625" style="3" customWidth="1"/>
-    <col min="4361" max="4361" width="26.5" style="3" customWidth="1"/>
-    <col min="4362" max="4362" width="34.1640625" style="3" customWidth="1"/>
+    <col min="4356" max="4356" width="17.109375" style="3" customWidth="1"/>
+    <col min="4357" max="4357" width="13.77734375" style="3" customWidth="1"/>
+    <col min="4358" max="4358" width="11.109375" style="3" customWidth="1"/>
+    <col min="4359" max="4359" width="23.44140625" style="3" customWidth="1"/>
+    <col min="4360" max="4360" width="44.109375" style="3" customWidth="1"/>
+    <col min="4361" max="4361" width="26.44140625" style="3" customWidth="1"/>
+    <col min="4362" max="4362" width="34.109375" style="3" customWidth="1"/>
     <col min="4363" max="4363" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="4364" max="4608" width="8.83203125" style="3"/>
+    <col min="4364" max="4608" width="8.77734375" style="3"/>
     <col min="4609" max="4609" width="2.33203125" style="3" customWidth="1"/>
     <col min="4610" max="4610" width="57.6640625" style="3" customWidth="1"/>
     <col min="4611" max="4611" width="18.6640625" style="3" customWidth="1"/>
-    <col min="4612" max="4612" width="17.1640625" style="3" customWidth="1"/>
-    <col min="4613" max="4613" width="13.83203125" style="3" customWidth="1"/>
-    <col min="4614" max="4614" width="11.1640625" style="3" customWidth="1"/>
-    <col min="4615" max="4615" width="23.5" style="3" customWidth="1"/>
-    <col min="4616" max="4616" width="44.1640625" style="3" customWidth="1"/>
-    <col min="4617" max="4617" width="26.5" style="3" customWidth="1"/>
-    <col min="4618" max="4618" width="34.1640625" style="3" customWidth="1"/>
+    <col min="4612" max="4612" width="17.109375" style="3" customWidth="1"/>
+    <col min="4613" max="4613" width="13.77734375" style="3" customWidth="1"/>
+    <col min="4614" max="4614" width="11.109375" style="3" customWidth="1"/>
+    <col min="4615" max="4615" width="23.44140625" style="3" customWidth="1"/>
+    <col min="4616" max="4616" width="44.109375" style="3" customWidth="1"/>
+    <col min="4617" max="4617" width="26.44140625" style="3" customWidth="1"/>
+    <col min="4618" max="4618" width="34.109375" style="3" customWidth="1"/>
     <col min="4619" max="4619" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="4620" max="4864" width="8.83203125" style="3"/>
+    <col min="4620" max="4864" width="8.77734375" style="3"/>
     <col min="4865" max="4865" width="2.33203125" style="3" customWidth="1"/>
     <col min="4866" max="4866" width="57.6640625" style="3" customWidth="1"/>
     <col min="4867" max="4867" width="18.6640625" style="3" customWidth="1"/>
-    <col min="4868" max="4868" width="17.1640625" style="3" customWidth="1"/>
-    <col min="4869" max="4869" width="13.83203125" style="3" customWidth="1"/>
-    <col min="4870" max="4870" width="11.1640625" style="3" customWidth="1"/>
-    <col min="4871" max="4871" width="23.5" style="3" customWidth="1"/>
-    <col min="4872" max="4872" width="44.1640625" style="3" customWidth="1"/>
-    <col min="4873" max="4873" width="26.5" style="3" customWidth="1"/>
-    <col min="4874" max="4874" width="34.1640625" style="3" customWidth="1"/>
+    <col min="4868" max="4868" width="17.109375" style="3" customWidth="1"/>
+    <col min="4869" max="4869" width="13.77734375" style="3" customWidth="1"/>
+    <col min="4870" max="4870" width="11.109375" style="3" customWidth="1"/>
+    <col min="4871" max="4871" width="23.44140625" style="3" customWidth="1"/>
+    <col min="4872" max="4872" width="44.109375" style="3" customWidth="1"/>
+    <col min="4873" max="4873" width="26.44140625" style="3" customWidth="1"/>
+    <col min="4874" max="4874" width="34.109375" style="3" customWidth="1"/>
     <col min="4875" max="4875" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="4876" max="5120" width="8.83203125" style="3"/>
+    <col min="4876" max="5120" width="8.77734375" style="3"/>
     <col min="5121" max="5121" width="2.33203125" style="3" customWidth="1"/>
     <col min="5122" max="5122" width="57.6640625" style="3" customWidth="1"/>
     <col min="5123" max="5123" width="18.6640625" style="3" customWidth="1"/>
-    <col min="5124" max="5124" width="17.1640625" style="3" customWidth="1"/>
-    <col min="5125" max="5125" width="13.83203125" style="3" customWidth="1"/>
-    <col min="5126" max="5126" width="11.1640625" style="3" customWidth="1"/>
-    <col min="5127" max="5127" width="23.5" style="3" customWidth="1"/>
-    <col min="5128" max="5128" width="44.1640625" style="3" customWidth="1"/>
-    <col min="5129" max="5129" width="26.5" style="3" customWidth="1"/>
-    <col min="5130" max="5130" width="34.1640625" style="3" customWidth="1"/>
+    <col min="5124" max="5124" width="17.109375" style="3" customWidth="1"/>
+    <col min="5125" max="5125" width="13.77734375" style="3" customWidth="1"/>
+    <col min="5126" max="5126" width="11.109375" style="3" customWidth="1"/>
+    <col min="5127" max="5127" width="23.44140625" style="3" customWidth="1"/>
+    <col min="5128" max="5128" width="44.109375" style="3" customWidth="1"/>
+    <col min="5129" max="5129" width="26.44140625" style="3" customWidth="1"/>
+    <col min="5130" max="5130" width="34.109375" style="3" customWidth="1"/>
     <col min="5131" max="5131" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="5132" max="5376" width="8.83203125" style="3"/>
+    <col min="5132" max="5376" width="8.77734375" style="3"/>
     <col min="5377" max="5377" width="2.33203125" style="3" customWidth="1"/>
     <col min="5378" max="5378" width="57.6640625" style="3" customWidth="1"/>
     <col min="5379" max="5379" width="18.6640625" style="3" customWidth="1"/>
-    <col min="5380" max="5380" width="17.1640625" style="3" customWidth="1"/>
-    <col min="5381" max="5381" width="13.83203125" style="3" customWidth="1"/>
-    <col min="5382" max="5382" width="11.1640625" style="3" customWidth="1"/>
-    <col min="5383" max="5383" width="23.5" style="3" customWidth="1"/>
-    <col min="5384" max="5384" width="44.1640625" style="3" customWidth="1"/>
-    <col min="5385" max="5385" width="26.5" style="3" customWidth="1"/>
-    <col min="5386" max="5386" width="34.1640625" style="3" customWidth="1"/>
+    <col min="5380" max="5380" width="17.109375" style="3" customWidth="1"/>
+    <col min="5381" max="5381" width="13.77734375" style="3" customWidth="1"/>
+    <col min="5382" max="5382" width="11.109375" style="3" customWidth="1"/>
+    <col min="5383" max="5383" width="23.44140625" style="3" customWidth="1"/>
+    <col min="5384" max="5384" width="44.109375" style="3" customWidth="1"/>
+    <col min="5385" max="5385" width="26.44140625" style="3" customWidth="1"/>
+    <col min="5386" max="5386" width="34.109375" style="3" customWidth="1"/>
     <col min="5387" max="5387" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="5388" max="5632" width="8.83203125" style="3"/>
+    <col min="5388" max="5632" width="8.77734375" style="3"/>
     <col min="5633" max="5633" width="2.33203125" style="3" customWidth="1"/>
     <col min="5634" max="5634" width="57.6640625" style="3" customWidth="1"/>
     <col min="5635" max="5635" width="18.6640625" style="3" customWidth="1"/>
-    <col min="5636" max="5636" width="17.1640625" style="3" customWidth="1"/>
-    <col min="5637" max="5637" width="13.83203125" style="3" customWidth="1"/>
-    <col min="5638" max="5638" width="11.1640625" style="3" customWidth="1"/>
-    <col min="5639" max="5639" width="23.5" style="3" customWidth="1"/>
-    <col min="5640" max="5640" width="44.1640625" style="3" customWidth="1"/>
-    <col min="5641" max="5641" width="26.5" style="3" customWidth="1"/>
-    <col min="5642" max="5642" width="34.1640625" style="3" customWidth="1"/>
+    <col min="5636" max="5636" width="17.109375" style="3" customWidth="1"/>
+    <col min="5637" max="5637" width="13.77734375" style="3" customWidth="1"/>
+    <col min="5638" max="5638" width="11.109375" style="3" customWidth="1"/>
+    <col min="5639" max="5639" width="23.44140625" style="3" customWidth="1"/>
+    <col min="5640" max="5640" width="44.109375" style="3" customWidth="1"/>
+    <col min="5641" max="5641" width="26.44140625" style="3" customWidth="1"/>
+    <col min="5642" max="5642" width="34.109375" style="3" customWidth="1"/>
     <col min="5643" max="5643" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="5644" max="5888" width="8.83203125" style="3"/>
+    <col min="5644" max="5888" width="8.77734375" style="3"/>
     <col min="5889" max="5889" width="2.33203125" style="3" customWidth="1"/>
     <col min="5890" max="5890" width="57.6640625" style="3" customWidth="1"/>
     <col min="5891" max="5891" width="18.6640625" style="3" customWidth="1"/>
-    <col min="5892" max="5892" width="17.1640625" style="3" customWidth="1"/>
-    <col min="5893" max="5893" width="13.83203125" style="3" customWidth="1"/>
-    <col min="5894" max="5894" width="11.1640625" style="3" customWidth="1"/>
-    <col min="5895" max="5895" width="23.5" style="3" customWidth="1"/>
-    <col min="5896" max="5896" width="44.1640625" style="3" customWidth="1"/>
-    <col min="5897" max="5897" width="26.5" style="3" customWidth="1"/>
-    <col min="5898" max="5898" width="34.1640625" style="3" customWidth="1"/>
+    <col min="5892" max="5892" width="17.109375" style="3" customWidth="1"/>
+    <col min="5893" max="5893" width="13.77734375" style="3" customWidth="1"/>
+    <col min="5894" max="5894" width="11.109375" style="3" customWidth="1"/>
+    <col min="5895" max="5895" width="23.44140625" style="3" customWidth="1"/>
+    <col min="5896" max="5896" width="44.109375" style="3" customWidth="1"/>
+    <col min="5897" max="5897" width="26.44140625" style="3" customWidth="1"/>
+    <col min="5898" max="5898" width="34.109375" style="3" customWidth="1"/>
     <col min="5899" max="5899" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="5900" max="6144" width="8.83203125" style="3"/>
+    <col min="5900" max="6144" width="8.77734375" style="3"/>
     <col min="6145" max="6145" width="2.33203125" style="3" customWidth="1"/>
     <col min="6146" max="6146" width="57.6640625" style="3" customWidth="1"/>
     <col min="6147" max="6147" width="18.6640625" style="3" customWidth="1"/>
-    <col min="6148" max="6148" width="17.1640625" style="3" customWidth="1"/>
-    <col min="6149" max="6149" width="13.83203125" style="3" customWidth="1"/>
-    <col min="6150" max="6150" width="11.1640625" style="3" customWidth="1"/>
-    <col min="6151" max="6151" width="23.5" style="3" customWidth="1"/>
-    <col min="6152" max="6152" width="44.1640625" style="3" customWidth="1"/>
-    <col min="6153" max="6153" width="26.5" style="3" customWidth="1"/>
-    <col min="6154" max="6154" width="34.1640625" style="3" customWidth="1"/>
+    <col min="6148" max="6148" width="17.109375" style="3" customWidth="1"/>
+    <col min="6149" max="6149" width="13.77734375" style="3" customWidth="1"/>
+    <col min="6150" max="6150" width="11.109375" style="3" customWidth="1"/>
+    <col min="6151" max="6151" width="23.44140625" style="3" customWidth="1"/>
+    <col min="6152" max="6152" width="44.109375" style="3" customWidth="1"/>
+    <col min="6153" max="6153" width="26.44140625" style="3" customWidth="1"/>
+    <col min="6154" max="6154" width="34.109375" style="3" customWidth="1"/>
     <col min="6155" max="6155" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="6156" max="6400" width="8.83203125" style="3"/>
+    <col min="6156" max="6400" width="8.77734375" style="3"/>
     <col min="6401" max="6401" width="2.33203125" style="3" customWidth="1"/>
     <col min="6402" max="6402" width="57.6640625" style="3" customWidth="1"/>
     <col min="6403" max="6403" width="18.6640625" style="3" customWidth="1"/>
-    <col min="6404" max="6404" width="17.1640625" style="3" customWidth="1"/>
-    <col min="6405" max="6405" width="13.83203125" style="3" customWidth="1"/>
-    <col min="6406" max="6406" width="11.1640625" style="3" customWidth="1"/>
-    <col min="6407" max="6407" width="23.5" style="3" customWidth="1"/>
-    <col min="6408" max="6408" width="44.1640625" style="3" customWidth="1"/>
-    <col min="6409" max="6409" width="26.5" style="3" customWidth="1"/>
-    <col min="6410" max="6410" width="34.1640625" style="3" customWidth="1"/>
+    <col min="6404" max="6404" width="17.109375" style="3" customWidth="1"/>
+    <col min="6405" max="6405" width="13.77734375" style="3" customWidth="1"/>
+    <col min="6406" max="6406" width="11.109375" style="3" customWidth="1"/>
+    <col min="6407" max="6407" width="23.44140625" style="3" customWidth="1"/>
+    <col min="6408" max="6408" width="44.109375" style="3" customWidth="1"/>
+    <col min="6409" max="6409" width="26.44140625" style="3" customWidth="1"/>
+    <col min="6410" max="6410" width="34.109375" style="3" customWidth="1"/>
     <col min="6411" max="6411" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="6412" max="6656" width="8.83203125" style="3"/>
+    <col min="6412" max="6656" width="8.77734375" style="3"/>
     <col min="6657" max="6657" width="2.33203125" style="3" customWidth="1"/>
     <col min="6658" max="6658" width="57.6640625" style="3" customWidth="1"/>
     <col min="6659" max="6659" width="18.6640625" style="3" customWidth="1"/>
-    <col min="6660" max="6660" width="17.1640625" style="3" customWidth="1"/>
-    <col min="6661" max="6661" width="13.83203125" style="3" customWidth="1"/>
-    <col min="6662" max="6662" width="11.1640625" style="3" customWidth="1"/>
-    <col min="6663" max="6663" width="23.5" style="3" customWidth="1"/>
-    <col min="6664" max="6664" width="44.1640625" style="3" customWidth="1"/>
-    <col min="6665" max="6665" width="26.5" style="3" customWidth="1"/>
-    <col min="6666" max="6666" width="34.1640625" style="3" customWidth="1"/>
+    <col min="6660" max="6660" width="17.109375" style="3" customWidth="1"/>
+    <col min="6661" max="6661" width="13.77734375" style="3" customWidth="1"/>
+    <col min="6662" max="6662" width="11.109375" style="3" customWidth="1"/>
+    <col min="6663" max="6663" width="23.44140625" style="3" customWidth="1"/>
+    <col min="6664" max="6664" width="44.109375" style="3" customWidth="1"/>
+    <col min="6665" max="6665" width="26.44140625" style="3" customWidth="1"/>
+    <col min="6666" max="6666" width="34.109375" style="3" customWidth="1"/>
     <col min="6667" max="6667" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="6668" max="6912" width="8.83203125" style="3"/>
+    <col min="6668" max="6912" width="8.77734375" style="3"/>
     <col min="6913" max="6913" width="2.33203125" style="3" customWidth="1"/>
     <col min="6914" max="6914" width="57.6640625" style="3" customWidth="1"/>
     <col min="6915" max="6915" width="18.6640625" style="3" customWidth="1"/>
-    <col min="6916" max="6916" width="17.1640625" style="3" customWidth="1"/>
-    <col min="6917" max="6917" width="13.83203125" style="3" customWidth="1"/>
-    <col min="6918" max="6918" width="11.1640625" style="3" customWidth="1"/>
-    <col min="6919" max="6919" width="23.5" style="3" customWidth="1"/>
-    <col min="6920" max="6920" width="44.1640625" style="3" customWidth="1"/>
-    <col min="6921" max="6921" width="26.5" style="3" customWidth="1"/>
-    <col min="6922" max="6922" width="34.1640625" style="3" customWidth="1"/>
+    <col min="6916" max="6916" width="17.109375" style="3" customWidth="1"/>
+    <col min="6917" max="6917" width="13.77734375" style="3" customWidth="1"/>
+    <col min="6918" max="6918" width="11.109375" style="3" customWidth="1"/>
+    <col min="6919" max="6919" width="23.44140625" style="3" customWidth="1"/>
+    <col min="6920" max="6920" width="44.109375" style="3" customWidth="1"/>
+    <col min="6921" max="6921" width="26.44140625" style="3" customWidth="1"/>
+    <col min="6922" max="6922" width="34.109375" style="3" customWidth="1"/>
     <col min="6923" max="6923" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="6924" max="7168" width="8.83203125" style="3"/>
+    <col min="6924" max="7168" width="8.77734375" style="3"/>
     <col min="7169" max="7169" width="2.33203125" style="3" customWidth="1"/>
     <col min="7170" max="7170" width="57.6640625" style="3" customWidth="1"/>
     <col min="7171" max="7171" width="18.6640625" style="3" customWidth="1"/>
-    <col min="7172" max="7172" width="17.1640625" style="3" customWidth="1"/>
-    <col min="7173" max="7173" width="13.83203125" style="3" customWidth="1"/>
-    <col min="7174" max="7174" width="11.1640625" style="3" customWidth="1"/>
-    <col min="7175" max="7175" width="23.5" style="3" customWidth="1"/>
-    <col min="7176" max="7176" width="44.1640625" style="3" customWidth="1"/>
-    <col min="7177" max="7177" width="26.5" style="3" customWidth="1"/>
-    <col min="7178" max="7178" width="34.1640625" style="3" customWidth="1"/>
+    <col min="7172" max="7172" width="17.109375" style="3" customWidth="1"/>
+    <col min="7173" max="7173" width="13.77734375" style="3" customWidth="1"/>
+    <col min="7174" max="7174" width="11.109375" style="3" customWidth="1"/>
+    <col min="7175" max="7175" width="23.44140625" style="3" customWidth="1"/>
+    <col min="7176" max="7176" width="44.109375" style="3" customWidth="1"/>
+    <col min="7177" max="7177" width="26.44140625" style="3" customWidth="1"/>
+    <col min="7178" max="7178" width="34.109375" style="3" customWidth="1"/>
     <col min="7179" max="7179" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="7180" max="7424" width="8.83203125" style="3"/>
+    <col min="7180" max="7424" width="8.77734375" style="3"/>
     <col min="7425" max="7425" width="2.33203125" style="3" customWidth="1"/>
     <col min="7426" max="7426" width="57.6640625" style="3" customWidth="1"/>
     <col min="7427" max="7427" width="18.6640625" style="3" customWidth="1"/>
-    <col min="7428" max="7428" width="17.1640625" style="3" customWidth="1"/>
-    <col min="7429" max="7429" width="13.83203125" style="3" customWidth="1"/>
-    <col min="7430" max="7430" width="11.1640625" style="3" customWidth="1"/>
-    <col min="7431" max="7431" width="23.5" style="3" customWidth="1"/>
-    <col min="7432" max="7432" width="44.1640625" style="3" customWidth="1"/>
-    <col min="7433" max="7433" width="26.5" style="3" customWidth="1"/>
-    <col min="7434" max="7434" width="34.1640625" style="3" customWidth="1"/>
+    <col min="7428" max="7428" width="17.109375" style="3" customWidth="1"/>
+    <col min="7429" max="7429" width="13.77734375" style="3" customWidth="1"/>
+    <col min="7430" max="7430" width="11.109375" style="3" customWidth="1"/>
+    <col min="7431" max="7431" width="23.44140625" style="3" customWidth="1"/>
+    <col min="7432" max="7432" width="44.109375" style="3" customWidth="1"/>
+    <col min="7433" max="7433" width="26.44140625" style="3" customWidth="1"/>
+    <col min="7434" max="7434" width="34.109375" style="3" customWidth="1"/>
     <col min="7435" max="7435" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="7436" max="7680" width="8.83203125" style="3"/>
+    <col min="7436" max="7680" width="8.77734375" style="3"/>
     <col min="7681" max="7681" width="2.33203125" style="3" customWidth="1"/>
     <col min="7682" max="7682" width="57.6640625" style="3" customWidth="1"/>
     <col min="7683" max="7683" width="18.6640625" style="3" customWidth="1"/>
-    <col min="7684" max="7684" width="17.1640625" style="3" customWidth="1"/>
-    <col min="7685" max="7685" width="13.83203125" style="3" customWidth="1"/>
-    <col min="7686" max="7686" width="11.1640625" style="3" customWidth="1"/>
-    <col min="7687" max="7687" width="23.5" style="3" customWidth="1"/>
-    <col min="7688" max="7688" width="44.1640625" style="3" customWidth="1"/>
-    <col min="7689" max="7689" width="26.5" style="3" customWidth="1"/>
-    <col min="7690" max="7690" width="34.1640625" style="3" customWidth="1"/>
+    <col min="7684" max="7684" width="17.109375" style="3" customWidth="1"/>
+    <col min="7685" max="7685" width="13.77734375" style="3" customWidth="1"/>
+    <col min="7686" max="7686" width="11.109375" style="3" customWidth="1"/>
+    <col min="7687" max="7687" width="23.44140625" style="3" customWidth="1"/>
+    <col min="7688" max="7688" width="44.109375" style="3" customWidth="1"/>
+    <col min="7689" max="7689" width="26.44140625" style="3" customWidth="1"/>
+    <col min="7690" max="7690" width="34.109375" style="3" customWidth="1"/>
     <col min="7691" max="7691" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="7692" max="7936" width="8.83203125" style="3"/>
+    <col min="7692" max="7936" width="8.77734375" style="3"/>
     <col min="7937" max="7937" width="2.33203125" style="3" customWidth="1"/>
     <col min="7938" max="7938" width="57.6640625" style="3" customWidth="1"/>
     <col min="7939" max="7939" width="18.6640625" style="3" customWidth="1"/>
-    <col min="7940" max="7940" width="17.1640625" style="3" customWidth="1"/>
-    <col min="7941" max="7941" width="13.83203125" style="3" customWidth="1"/>
-    <col min="7942" max="7942" width="11.1640625" style="3" customWidth="1"/>
-    <col min="7943" max="7943" width="23.5" style="3" customWidth="1"/>
-    <col min="7944" max="7944" width="44.1640625" style="3" customWidth="1"/>
-    <col min="7945" max="7945" width="26.5" style="3" customWidth="1"/>
-    <col min="7946" max="7946" width="34.1640625" style="3" customWidth="1"/>
+    <col min="7940" max="7940" width="17.109375" style="3" customWidth="1"/>
+    <col min="7941" max="7941" width="13.77734375" style="3" customWidth="1"/>
+    <col min="7942" max="7942" width="11.109375" style="3" customWidth="1"/>
+    <col min="7943" max="7943" width="23.44140625" style="3" customWidth="1"/>
+    <col min="7944" max="7944" width="44.109375" style="3" customWidth="1"/>
+    <col min="7945" max="7945" width="26.44140625" style="3" customWidth="1"/>
+    <col min="7946" max="7946" width="34.109375" style="3" customWidth="1"/>
     <col min="7947" max="7947" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="7948" max="8192" width="8.83203125" style="3"/>
+    <col min="7948" max="8192" width="8.77734375" style="3"/>
     <col min="8193" max="8193" width="2.33203125" style="3" customWidth="1"/>
     <col min="8194" max="8194" width="57.6640625" style="3" customWidth="1"/>
     <col min="8195" max="8195" width="18.6640625" style="3" customWidth="1"/>
-    <col min="8196" max="8196" width="17.1640625" style="3" customWidth="1"/>
-    <col min="8197" max="8197" width="13.83203125" style="3" customWidth="1"/>
-    <col min="8198" max="8198" width="11.1640625" style="3" customWidth="1"/>
-    <col min="8199" max="8199" width="23.5" style="3" customWidth="1"/>
-    <col min="8200" max="8200" width="44.1640625" style="3" customWidth="1"/>
-    <col min="8201" max="8201" width="26.5" style="3" customWidth="1"/>
-    <col min="8202" max="8202" width="34.1640625" style="3" customWidth="1"/>
+    <col min="8196" max="8196" width="17.109375" style="3" customWidth="1"/>
+    <col min="8197" max="8197" width="13.77734375" style="3" customWidth="1"/>
+    <col min="8198" max="8198" width="11.109375" style="3" customWidth="1"/>
+    <col min="8199" max="8199" width="23.44140625" style="3" customWidth="1"/>
+    <col min="8200" max="8200" width="44.109375" style="3" customWidth="1"/>
+    <col min="8201" max="8201" width="26.44140625" style="3" customWidth="1"/>
+    <col min="8202" max="8202" width="34.109375" style="3" customWidth="1"/>
     <col min="8203" max="8203" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="8204" max="8448" width="8.83203125" style="3"/>
+    <col min="8204" max="8448" width="8.77734375" style="3"/>
     <col min="8449" max="8449" width="2.33203125" style="3" customWidth="1"/>
     <col min="8450" max="8450" width="57.6640625" style="3" customWidth="1"/>
     <col min="8451" max="8451" width="18.6640625" style="3" customWidth="1"/>
-    <col min="8452" max="8452" width="17.1640625" style="3" customWidth="1"/>
-    <col min="8453" max="8453" width="13.83203125" style="3" customWidth="1"/>
-    <col min="8454" max="8454" width="11.1640625" style="3" customWidth="1"/>
-    <col min="8455" max="8455" width="23.5" style="3" customWidth="1"/>
-    <col min="8456" max="8456" width="44.1640625" style="3" customWidth="1"/>
-    <col min="8457" max="8457" width="26.5" style="3" customWidth="1"/>
-    <col min="8458" max="8458" width="34.1640625" style="3" customWidth="1"/>
+    <col min="8452" max="8452" width="17.109375" style="3" customWidth="1"/>
+    <col min="8453" max="8453" width="13.77734375" style="3" customWidth="1"/>
+    <col min="8454" max="8454" width="11.109375" style="3" customWidth="1"/>
+    <col min="8455" max="8455" width="23.44140625" style="3" customWidth="1"/>
+    <col min="8456" max="8456" width="44.109375" style="3" customWidth="1"/>
+    <col min="8457" max="8457" width="26.44140625" style="3" customWidth="1"/>
+    <col min="8458" max="8458" width="34.109375" style="3" customWidth="1"/>
     <col min="8459" max="8459" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="8460" max="8704" width="8.83203125" style="3"/>
+    <col min="8460" max="8704" width="8.77734375" style="3"/>
     <col min="8705" max="8705" width="2.33203125" style="3" customWidth="1"/>
     <col min="8706" max="8706" width="57.6640625" style="3" customWidth="1"/>
     <col min="8707" max="8707" width="18.6640625" style="3" customWidth="1"/>
-    <col min="8708" max="8708" width="17.1640625" style="3" customWidth="1"/>
-    <col min="8709" max="8709" width="13.83203125" style="3" customWidth="1"/>
-    <col min="8710" max="8710" width="11.1640625" style="3" customWidth="1"/>
-    <col min="8711" max="8711" width="23.5" style="3" customWidth="1"/>
-    <col min="8712" max="8712" width="44.1640625" style="3" customWidth="1"/>
-    <col min="8713" max="8713" width="26.5" style="3" customWidth="1"/>
-    <col min="8714" max="8714" width="34.1640625" style="3" customWidth="1"/>
+    <col min="8708" max="8708" width="17.109375" style="3" customWidth="1"/>
+    <col min="8709" max="8709" width="13.77734375" style="3" customWidth="1"/>
+    <col min="8710" max="8710" width="11.109375" style="3" customWidth="1"/>
+    <col min="8711" max="8711" width="23.44140625" style="3" customWidth="1"/>
+    <col min="8712" max="8712" width="44.109375" style="3" customWidth="1"/>
+    <col min="8713" max="8713" width="26.44140625" style="3" customWidth="1"/>
+    <col min="8714" max="8714" width="34.109375" style="3" customWidth="1"/>
     <col min="8715" max="8715" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="8716" max="8960" width="8.83203125" style="3"/>
+    <col min="8716" max="8960" width="8.77734375" style="3"/>
     <col min="8961" max="8961" width="2.33203125" style="3" customWidth="1"/>
     <col min="8962" max="8962" width="57.6640625" style="3" customWidth="1"/>
     <col min="8963" max="8963" width="18.6640625" style="3" customWidth="1"/>
-    <col min="8964" max="8964" width="17.1640625" style="3" customWidth="1"/>
-    <col min="8965" max="8965" width="13.83203125" style="3" customWidth="1"/>
-    <col min="8966" max="8966" width="11.1640625" style="3" customWidth="1"/>
-    <col min="8967" max="8967" width="23.5" style="3" customWidth="1"/>
-    <col min="8968" max="8968" width="44.1640625" style="3" customWidth="1"/>
-    <col min="8969" max="8969" width="26.5" style="3" customWidth="1"/>
-    <col min="8970" max="8970" width="34.1640625" style="3" customWidth="1"/>
+    <col min="8964" max="8964" width="17.109375" style="3" customWidth="1"/>
+    <col min="8965" max="8965" width="13.77734375" style="3" customWidth="1"/>
+    <col min="8966" max="8966" width="11.109375" style="3" customWidth="1"/>
+    <col min="8967" max="8967" width="23.44140625" style="3" customWidth="1"/>
+    <col min="8968" max="8968" width="44.109375" style="3" customWidth="1"/>
+    <col min="8969" max="8969" width="26.44140625" style="3" customWidth="1"/>
+    <col min="8970" max="8970" width="34.109375" style="3" customWidth="1"/>
     <col min="8971" max="8971" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="8972" max="9216" width="8.83203125" style="3"/>
+    <col min="8972" max="9216" width="8.77734375" style="3"/>
     <col min="9217" max="9217" width="2.33203125" style="3" customWidth="1"/>
     <col min="9218" max="9218" width="57.6640625" style="3" customWidth="1"/>
     <col min="9219" max="9219" width="18.6640625" style="3" customWidth="1"/>
-    <col min="9220" max="9220" width="17.1640625" style="3" customWidth="1"/>
-    <col min="9221" max="9221" width="13.83203125" style="3" customWidth="1"/>
-    <col min="9222" max="9222" width="11.1640625" style="3" customWidth="1"/>
-    <col min="9223" max="9223" width="23.5" style="3" customWidth="1"/>
-    <col min="9224" max="9224" width="44.1640625" style="3" customWidth="1"/>
-    <col min="9225" max="9225" width="26.5" style="3" customWidth="1"/>
-    <col min="9226" max="9226" width="34.1640625" style="3" customWidth="1"/>
+    <col min="9220" max="9220" width="17.109375" style="3" customWidth="1"/>
+    <col min="9221" max="9221" width="13.77734375" style="3" customWidth="1"/>
+    <col min="9222" max="9222" width="11.109375" style="3" customWidth="1"/>
+    <col min="9223" max="9223" width="23.44140625" style="3" customWidth="1"/>
+    <col min="9224" max="9224" width="44.109375" style="3" customWidth="1"/>
+    <col min="9225" max="9225" width="26.44140625" style="3" customWidth="1"/>
+    <col min="9226" max="9226" width="34.109375" style="3" customWidth="1"/>
     <col min="9227" max="9227" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="9228" max="9472" width="8.83203125" style="3"/>
+    <col min="9228" max="9472" width="8.77734375" style="3"/>
     <col min="9473" max="9473" width="2.33203125" style="3" customWidth="1"/>
     <col min="9474" max="9474" width="57.6640625" style="3" customWidth="1"/>
     <col min="9475" max="9475" width="18.6640625" style="3" customWidth="1"/>
-    <col min="9476" max="9476" width="17.1640625" style="3" customWidth="1"/>
-    <col min="9477" max="9477" width="13.83203125" style="3" customWidth="1"/>
-    <col min="9478" max="9478" width="11.1640625" style="3" customWidth="1"/>
-    <col min="9479" max="9479" width="23.5" style="3" customWidth="1"/>
-    <col min="9480" max="9480" width="44.1640625" style="3" customWidth="1"/>
-    <col min="9481" max="9481" width="26.5" style="3" customWidth="1"/>
-    <col min="9482" max="9482" width="34.1640625" style="3" customWidth="1"/>
+    <col min="9476" max="9476" width="17.109375" style="3" customWidth="1"/>
+    <col min="9477" max="9477" width="13.77734375" style="3" customWidth="1"/>
+    <col min="9478" max="9478" width="11.109375" style="3" customWidth="1"/>
+    <col min="9479" max="9479" width="23.44140625" style="3" customWidth="1"/>
+    <col min="9480" max="9480" width="44.109375" style="3" customWidth="1"/>
+    <col min="9481" max="9481" width="26.44140625" style="3" customWidth="1"/>
+    <col min="9482" max="9482" width="34.109375" style="3" customWidth="1"/>
     <col min="9483" max="9483" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="9484" max="9728" width="8.83203125" style="3"/>
+    <col min="9484" max="9728" width="8.77734375" style="3"/>
     <col min="9729" max="9729" width="2.33203125" style="3" customWidth="1"/>
     <col min="9730" max="9730" width="57.6640625" style="3" customWidth="1"/>
     <col min="9731" max="9731" width="18.6640625" style="3" customWidth="1"/>
-    <col min="9732" max="9732" width="17.1640625" style="3" customWidth="1"/>
-    <col min="9733" max="9733" width="13.83203125" style="3" customWidth="1"/>
-    <col min="9734" max="9734" width="11.1640625" style="3" customWidth="1"/>
-    <col min="9735" max="9735" width="23.5" style="3" customWidth="1"/>
-    <col min="9736" max="9736" width="44.1640625" style="3" customWidth="1"/>
-    <col min="9737" max="9737" width="26.5" style="3" customWidth="1"/>
-    <col min="9738" max="9738" width="34.1640625" style="3" customWidth="1"/>
+    <col min="9732" max="9732" width="17.109375" style="3" customWidth="1"/>
+    <col min="9733" max="9733" width="13.77734375" style="3" customWidth="1"/>
+    <col min="9734" max="9734" width="11.109375" style="3" customWidth="1"/>
+    <col min="9735" max="9735" width="23.44140625" style="3" customWidth="1"/>
+    <col min="9736" max="9736" width="44.109375" style="3" customWidth="1"/>
+    <col min="9737" max="9737" width="26.44140625" style="3" customWidth="1"/>
+    <col min="9738" max="9738" width="34.109375" style="3" customWidth="1"/>
     <col min="9739" max="9739" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="9740" max="9984" width="8.83203125" style="3"/>
+    <col min="9740" max="9984" width="8.77734375" style="3"/>
     <col min="9985" max="9985" width="2.33203125" style="3" customWidth="1"/>
     <col min="9986" max="9986" width="57.6640625" style="3" customWidth="1"/>
     <col min="9987" max="9987" width="18.6640625" style="3" customWidth="1"/>
-    <col min="9988" max="9988" width="17.1640625" style="3" customWidth="1"/>
-    <col min="9989" max="9989" width="13.83203125" style="3" customWidth="1"/>
-    <col min="9990" max="9990" width="11.1640625" style="3" customWidth="1"/>
-    <col min="9991" max="9991" width="23.5" style="3" customWidth="1"/>
-    <col min="9992" max="9992" width="44.1640625" style="3" customWidth="1"/>
-    <col min="9993" max="9993" width="26.5" style="3" customWidth="1"/>
-    <col min="9994" max="9994" width="34.1640625" style="3" customWidth="1"/>
+    <col min="9988" max="9988" width="17.109375" style="3" customWidth="1"/>
+    <col min="9989" max="9989" width="13.77734375" style="3" customWidth="1"/>
+    <col min="9990" max="9990" width="11.109375" style="3" customWidth="1"/>
+    <col min="9991" max="9991" width="23.44140625" style="3" customWidth="1"/>
+    <col min="9992" max="9992" width="44.109375" style="3" customWidth="1"/>
+    <col min="9993" max="9993" width="26.44140625" style="3" customWidth="1"/>
+    <col min="9994" max="9994" width="34.109375" style="3" customWidth="1"/>
     <col min="9995" max="9995" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="9996" max="10240" width="8.83203125" style="3"/>
+    <col min="9996" max="10240" width="8.77734375" style="3"/>
     <col min="10241" max="10241" width="2.33203125" style="3" customWidth="1"/>
     <col min="10242" max="10242" width="57.6640625" style="3" customWidth="1"/>
     <col min="10243" max="10243" width="18.6640625" style="3" customWidth="1"/>
-    <col min="10244" max="10244" width="17.1640625" style="3" customWidth="1"/>
-    <col min="10245" max="10245" width="13.83203125" style="3" customWidth="1"/>
-    <col min="10246" max="10246" width="11.1640625" style="3" customWidth="1"/>
-    <col min="10247" max="10247" width="23.5" style="3" customWidth="1"/>
-    <col min="10248" max="10248" width="44.1640625" style="3" customWidth="1"/>
-    <col min="10249" max="10249" width="26.5" style="3" customWidth="1"/>
-    <col min="10250" max="10250" width="34.1640625" style="3" customWidth="1"/>
+    <col min="10244" max="10244" width="17.109375" style="3" customWidth="1"/>
+    <col min="10245" max="10245" width="13.77734375" style="3" customWidth="1"/>
+    <col min="10246" max="10246" width="11.109375" style="3" customWidth="1"/>
+    <col min="10247" max="10247" width="23.44140625" style="3" customWidth="1"/>
+    <col min="10248" max="10248" width="44.109375" style="3" customWidth="1"/>
+    <col min="10249" max="10249" width="26.44140625" style="3" customWidth="1"/>
+    <col min="10250" max="10250" width="34.109375" style="3" customWidth="1"/>
     <col min="10251" max="10251" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="10252" max="10496" width="8.83203125" style="3"/>
+    <col min="10252" max="10496" width="8.77734375" style="3"/>
     <col min="10497" max="10497" width="2.33203125" style="3" customWidth="1"/>
     <col min="10498" max="10498" width="57.6640625" style="3" customWidth="1"/>
     <col min="10499" max="10499" width="18.6640625" style="3" customWidth="1"/>
-    <col min="10500" max="10500" width="17.1640625" style="3" customWidth="1"/>
-    <col min="10501" max="10501" width="13.83203125" style="3" customWidth="1"/>
-    <col min="10502" max="10502" width="11.1640625" style="3" customWidth="1"/>
-    <col min="10503" max="10503" width="23.5" style="3" customWidth="1"/>
-    <col min="10504" max="10504" width="44.1640625" style="3" customWidth="1"/>
-    <col min="10505" max="10505" width="26.5" style="3" customWidth="1"/>
-    <col min="10506" max="10506" width="34.1640625" style="3" customWidth="1"/>
+    <col min="10500" max="10500" width="17.109375" style="3" customWidth="1"/>
+    <col min="10501" max="10501" width="13.77734375" style="3" customWidth="1"/>
+    <col min="10502" max="10502" width="11.109375" style="3" customWidth="1"/>
+    <col min="10503" max="10503" width="23.44140625" style="3" customWidth="1"/>
+    <col min="10504" max="10504" width="44.109375" style="3" customWidth="1"/>
+    <col min="10505" max="10505" width="26.44140625" style="3" customWidth="1"/>
+    <col min="10506" max="10506" width="34.109375" style="3" customWidth="1"/>
     <col min="10507" max="10507" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="10508" max="10752" width="8.83203125" style="3"/>
+    <col min="10508" max="10752" width="8.77734375" style="3"/>
     <col min="10753" max="10753" width="2.33203125" style="3" customWidth="1"/>
     <col min="10754" max="10754" width="57.6640625" style="3" customWidth="1"/>
     <col min="10755" max="10755" width="18.6640625" style="3" customWidth="1"/>
-    <col min="10756" max="10756" width="17.1640625" style="3" customWidth="1"/>
-    <col min="10757" max="10757" width="13.83203125" style="3" customWidth="1"/>
-    <col min="10758" max="10758" width="11.1640625" style="3" customWidth="1"/>
-    <col min="10759" max="10759" width="23.5" style="3" customWidth="1"/>
-    <col min="10760" max="10760" width="44.1640625" style="3" customWidth="1"/>
-    <col min="10761" max="10761" width="26.5" style="3" customWidth="1"/>
-    <col min="10762" max="10762" width="34.1640625" style="3" customWidth="1"/>
+    <col min="10756" max="10756" width="17.109375" style="3" customWidth="1"/>
+    <col min="10757" max="10757" width="13.77734375" style="3" customWidth="1"/>
+    <col min="10758" max="10758" width="11.109375" style="3" customWidth="1"/>
+    <col min="10759" max="10759" width="23.44140625" style="3" customWidth="1"/>
+    <col min="10760" max="10760" width="44.109375" style="3" customWidth="1"/>
+    <col min="10761" max="10761" width="26.44140625" style="3" customWidth="1"/>
+    <col min="10762" max="10762" width="34.109375" style="3" customWidth="1"/>
     <col min="10763" max="10763" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="10764" max="11008" width="8.83203125" style="3"/>
+    <col min="10764" max="11008" width="8.77734375" style="3"/>
     <col min="11009" max="11009" width="2.33203125" style="3" customWidth="1"/>
     <col min="11010" max="11010" width="57.6640625" style="3" customWidth="1"/>
     <col min="11011" max="11011" width="18.6640625" style="3" customWidth="1"/>
-    <col min="11012" max="11012" width="17.1640625" style="3" customWidth="1"/>
-    <col min="11013" max="11013" width="13.83203125" style="3" customWidth="1"/>
-    <col min="11014" max="11014" width="11.1640625" style="3" customWidth="1"/>
-    <col min="11015" max="11015" width="23.5" style="3" customWidth="1"/>
-    <col min="11016" max="11016" width="44.1640625" style="3" customWidth="1"/>
-    <col min="11017" max="11017" width="26.5" style="3" customWidth="1"/>
-    <col min="11018" max="11018" width="34.1640625" style="3" customWidth="1"/>
+    <col min="11012" max="11012" width="17.109375" style="3" customWidth="1"/>
+    <col min="11013" max="11013" width="13.77734375" style="3" customWidth="1"/>
+    <col min="11014" max="11014" width="11.109375" style="3" customWidth="1"/>
+    <col min="11015" max="11015" width="23.44140625" style="3" customWidth="1"/>
+    <col min="11016" max="11016" width="44.109375" style="3" customWidth="1"/>
+    <col min="11017" max="11017" width="26.44140625" style="3" customWidth="1"/>
+    <col min="11018" max="11018" width="34.109375" style="3" customWidth="1"/>
     <col min="11019" max="11019" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="11020" max="11264" width="8.83203125" style="3"/>
+    <col min="11020" max="11264" width="8.77734375" style="3"/>
     <col min="11265" max="11265" width="2.33203125" style="3" customWidth="1"/>
     <col min="11266" max="11266" width="57.6640625" style="3" customWidth="1"/>
     <col min="11267" max="11267" width="18.6640625" style="3" customWidth="1"/>
-    <col min="11268" max="11268" width="17.1640625" style="3" customWidth="1"/>
-    <col min="11269" max="11269" width="13.83203125" style="3" customWidth="1"/>
-    <col min="11270" max="11270" width="11.1640625" style="3" customWidth="1"/>
-    <col min="11271" max="11271" width="23.5" style="3" customWidth="1"/>
-    <col min="11272" max="11272" width="44.1640625" style="3" customWidth="1"/>
-    <col min="11273" max="11273" width="26.5" style="3" customWidth="1"/>
-    <col min="11274" max="11274" width="34.1640625" style="3" customWidth="1"/>
+    <col min="11268" max="11268" width="17.109375" style="3" customWidth="1"/>
+    <col min="11269" max="11269" width="13.77734375" style="3" customWidth="1"/>
+    <col min="11270" max="11270" width="11.109375" style="3" customWidth="1"/>
+    <col min="11271" max="11271" width="23.44140625" style="3" customWidth="1"/>
+    <col min="11272" max="11272" width="44.109375" style="3" customWidth="1"/>
+    <col min="11273" max="11273" width="26.44140625" style="3" customWidth="1"/>
+    <col min="11274" max="11274" width="34.109375" style="3" customWidth="1"/>
     <col min="11275" max="11275" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="11276" max="11520" width="8.83203125" style="3"/>
+    <col min="11276" max="11520" width="8.77734375" style="3"/>
     <col min="11521" max="11521" width="2.33203125" style="3" customWidth="1"/>
     <col min="11522" max="11522" width="57.6640625" style="3" customWidth="1"/>
     <col min="11523" max="11523" width="18.6640625" style="3" customWidth="1"/>
-    <col min="11524" max="11524" width="17.1640625" style="3" customWidth="1"/>
-    <col min="11525" max="11525" width="13.83203125" style="3" customWidth="1"/>
-    <col min="11526" max="11526" width="11.1640625" style="3" customWidth="1"/>
-    <col min="11527" max="11527" width="23.5" style="3" customWidth="1"/>
-    <col min="11528" max="11528" width="44.1640625" style="3" customWidth="1"/>
-    <col min="11529" max="11529" width="26.5" style="3" customWidth="1"/>
-    <col min="11530" max="11530" width="34.1640625" style="3" customWidth="1"/>
+    <col min="11524" max="11524" width="17.109375" style="3" customWidth="1"/>
+    <col min="11525" max="11525" width="13.77734375" style="3" customWidth="1"/>
+    <col min="11526" max="11526" width="11.109375" style="3" customWidth="1"/>
+    <col min="11527" max="11527" width="23.44140625" style="3" customWidth="1"/>
+    <col min="11528" max="11528" width="44.109375" style="3" customWidth="1"/>
+    <col min="11529" max="11529" width="26.44140625" style="3" customWidth="1"/>
+    <col min="11530" max="11530" width="34.109375" style="3" customWidth="1"/>
     <col min="11531" max="11531" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="11532" max="11776" width="8.83203125" style="3"/>
+    <col min="11532" max="11776" width="8.77734375" style="3"/>
     <col min="11777" max="11777" width="2.33203125" style="3" customWidth="1"/>
     <col min="11778" max="11778" width="57.6640625" style="3" customWidth="1"/>
     <col min="11779" max="11779" width="18.6640625" style="3" customWidth="1"/>
-    <col min="11780" max="11780" width="17.1640625" style="3" customWidth="1"/>
-    <col min="11781" max="11781" width="13.83203125" style="3" customWidth="1"/>
-    <col min="11782" max="11782" width="11.1640625" style="3" customWidth="1"/>
-    <col min="11783" max="11783" width="23.5" style="3" customWidth="1"/>
-    <col min="11784" max="11784" width="44.1640625" style="3" customWidth="1"/>
-    <col min="11785" max="11785" width="26.5" style="3" customWidth="1"/>
-    <col min="11786" max="11786" width="34.1640625" style="3" customWidth="1"/>
+    <col min="11780" max="11780" width="17.109375" style="3" customWidth="1"/>
+    <col min="11781" max="11781" width="13.77734375" style="3" customWidth="1"/>
+    <col min="11782" max="11782" width="11.109375" style="3" customWidth="1"/>
+    <col min="11783" max="11783" width="23.44140625" style="3" customWidth="1"/>
+    <col min="11784" max="11784" width="44.109375" style="3" customWidth="1"/>
+    <col min="11785" max="11785" width="26.44140625" style="3" customWidth="1"/>
+    <col min="11786" max="11786" width="34.109375" style="3" customWidth="1"/>
     <col min="11787" max="11787" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="11788" max="12032" width="8.83203125" style="3"/>
+    <col min="11788" max="12032" width="8.77734375" style="3"/>
     <col min="12033" max="12033" width="2.33203125" style="3" customWidth="1"/>
     <col min="12034" max="12034" width="57.6640625" style="3" customWidth="1"/>
     <col min="12035" max="12035" width="18.6640625" style="3" customWidth="1"/>
-    <col min="12036" max="12036" width="17.1640625" style="3" customWidth="1"/>
-    <col min="12037" max="12037" width="13.83203125" style="3" customWidth="1"/>
-    <col min="12038" max="12038" width="11.1640625" style="3" customWidth="1"/>
-    <col min="12039" max="12039" width="23.5" style="3" customWidth="1"/>
-    <col min="12040" max="12040" width="44.1640625" style="3" customWidth="1"/>
-    <col min="12041" max="12041" width="26.5" style="3" customWidth="1"/>
-    <col min="12042" max="12042" width="34.1640625" style="3" customWidth="1"/>
+    <col min="12036" max="12036" width="17.109375" style="3" customWidth="1"/>
+    <col min="12037" max="12037" width="13.77734375" style="3" customWidth="1"/>
+    <col min="12038" max="12038" width="11.109375" style="3" customWidth="1"/>
+    <col min="12039" max="12039" width="23.44140625" style="3" customWidth="1"/>
+    <col min="12040" max="12040" width="44.109375" style="3" customWidth="1"/>
+    <col min="12041" max="12041" width="26.44140625" style="3" customWidth="1"/>
+    <col min="12042" max="12042" width="34.109375" style="3" customWidth="1"/>
     <col min="12043" max="12043" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="12044" max="12288" width="8.83203125" style="3"/>
+    <col min="12044" max="12288" width="8.77734375" style="3"/>
     <col min="12289" max="12289" width="2.33203125" style="3" customWidth="1"/>
     <col min="12290" max="12290" width="57.6640625" style="3" customWidth="1"/>
     <col min="12291" max="12291" width="18.6640625" style="3" customWidth="1"/>
-    <col min="12292" max="12292" width="17.1640625" style="3" customWidth="1"/>
-    <col min="12293" max="12293" width="13.83203125" style="3" customWidth="1"/>
-    <col min="12294" max="12294" width="11.1640625" style="3" customWidth="1"/>
-    <col min="12295" max="12295" width="23.5" style="3" customWidth="1"/>
-    <col min="12296" max="12296" width="44.1640625" style="3" customWidth="1"/>
-    <col min="12297" max="12297" width="26.5" style="3" customWidth="1"/>
-    <col min="12298" max="12298" width="34.1640625" style="3" customWidth="1"/>
+    <col min="12292" max="12292" width="17.109375" style="3" customWidth="1"/>
+    <col min="12293" max="12293" width="13.77734375" style="3" customWidth="1"/>
+    <col min="12294" max="12294" width="11.109375" style="3" customWidth="1"/>
+    <col min="12295" max="12295" width="23.44140625" style="3" customWidth="1"/>
+    <col min="12296" max="12296" width="44.109375" style="3" customWidth="1"/>
+    <col min="12297" max="12297" width="26.44140625" style="3" customWidth="1"/>
+    <col min="12298" max="12298" width="34.109375" style="3" customWidth="1"/>
     <col min="12299" max="12299" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="12300" max="12544" width="8.83203125" style="3"/>
+    <col min="12300" max="12544" width="8.77734375" style="3"/>
     <col min="12545" max="12545" width="2.33203125" style="3" customWidth="1"/>
     <col min="12546" max="12546" width="57.6640625" style="3" customWidth="1"/>
     <col min="12547" max="12547" width="18.6640625" style="3" customWidth="1"/>
-    <col min="12548" max="12548" width="17.1640625" style="3" customWidth="1"/>
-    <col min="12549" max="12549" width="13.83203125" style="3" customWidth="1"/>
-    <col min="12550" max="12550" width="11.1640625" style="3" customWidth="1"/>
-    <col min="12551" max="12551" width="23.5" style="3" customWidth="1"/>
-    <col min="12552" max="12552" width="44.1640625" style="3" customWidth="1"/>
-    <col min="12553" max="12553" width="26.5" style="3" customWidth="1"/>
-    <col min="12554" max="12554" width="34.1640625" style="3" customWidth="1"/>
+    <col min="12548" max="12548" width="17.109375" style="3" customWidth="1"/>
+    <col min="12549" max="12549" width="13.77734375" style="3" customWidth="1"/>
+    <col min="12550" max="12550" width="11.109375" style="3" customWidth="1"/>
+    <col min="12551" max="12551" width="23.44140625" style="3" customWidth="1"/>
+    <col min="12552" max="12552" width="44.109375" style="3" customWidth="1"/>
+    <col min="12553" max="12553" width="26.44140625" style="3" customWidth="1"/>
+    <col min="12554" max="12554" width="34.109375" style="3" customWidth="1"/>
     <col min="12555" max="12555" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="12556" max="12800" width="8.83203125" style="3"/>
+    <col min="12556" max="12800" width="8.77734375" style="3"/>
     <col min="12801" max="12801" width="2.33203125" style="3" customWidth="1"/>
     <col min="12802" max="12802" width="57.6640625" style="3" customWidth="1"/>
     <col min="12803" max="12803" width="18.6640625" style="3" customWidth="1"/>
-    <col min="12804" max="12804" width="17.1640625" style="3" customWidth="1"/>
-    <col min="12805" max="12805" width="13.83203125" style="3" customWidth="1"/>
-    <col min="12806" max="12806" width="11.1640625" style="3" customWidth="1"/>
-    <col min="12807" max="12807" width="23.5" style="3" customWidth="1"/>
-    <col min="12808" max="12808" width="44.1640625" style="3" customWidth="1"/>
-    <col min="12809" max="12809" width="26.5" style="3" customWidth="1"/>
-    <col min="12810" max="12810" width="34.1640625" style="3" customWidth="1"/>
+    <col min="12804" max="12804" width="17.109375" style="3" customWidth="1"/>
+    <col min="12805" max="12805" width="13.77734375" style="3" customWidth="1"/>
+    <col min="12806" max="12806" width="11.109375" style="3" customWidth="1"/>
+    <col min="12807" max="12807" width="23.44140625" style="3" customWidth="1"/>
+    <col min="12808" max="12808" width="44.109375" style="3" customWidth="1"/>
+    <col min="12809" max="12809" width="26.44140625" style="3" customWidth="1"/>
+    <col min="12810" max="12810" width="34.109375" style="3" customWidth="1"/>
     <col min="12811" max="12811" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="12812" max="13056" width="8.83203125" style="3"/>
+    <col min="12812" max="13056" width="8.77734375" style="3"/>
     <col min="13057" max="13057" width="2.33203125" style="3" customWidth="1"/>
     <col min="13058" max="13058" width="57.6640625" style="3" customWidth="1"/>
     <col min="13059" max="13059" width="18.6640625" style="3" customWidth="1"/>
-    <col min="13060" max="13060" width="17.1640625" style="3" customWidth="1"/>
-    <col min="13061" max="13061" width="13.83203125" style="3" customWidth="1"/>
-    <col min="13062" max="13062" width="11.1640625" style="3" customWidth="1"/>
-    <col min="13063" max="13063" width="23.5" style="3" customWidth="1"/>
-    <col min="13064" max="13064" width="44.1640625" style="3" customWidth="1"/>
-    <col min="13065" max="13065" width="26.5" style="3" customWidth="1"/>
-    <col min="13066" max="13066" width="34.1640625" style="3" customWidth="1"/>
+    <col min="13060" max="13060" width="17.109375" style="3" customWidth="1"/>
+    <col min="13061" max="13061" width="13.77734375" style="3" customWidth="1"/>
+    <col min="13062" max="13062" width="11.109375" style="3" customWidth="1"/>
+    <col min="13063" max="13063" width="23.44140625" style="3" customWidth="1"/>
+    <col min="13064" max="13064" width="44.109375" style="3" customWidth="1"/>
+    <col min="13065" max="13065" width="26.44140625" style="3" customWidth="1"/>
+    <col min="13066" max="13066" width="34.109375" style="3" customWidth="1"/>
     <col min="13067" max="13067" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="13068" max="13312" width="8.83203125" style="3"/>
+    <col min="13068" max="13312" width="8.77734375" style="3"/>
     <col min="13313" max="13313" width="2.33203125" style="3" customWidth="1"/>
     <col min="13314" max="13314" width="57.6640625" style="3" customWidth="1"/>
     <col min="13315" max="13315" width="18.6640625" style="3" customWidth="1"/>
-    <col min="13316" max="13316" width="17.1640625" style="3" customWidth="1"/>
-    <col min="13317" max="13317" width="13.83203125" style="3" customWidth="1"/>
-    <col min="13318" max="13318" width="11.1640625" style="3" customWidth="1"/>
-    <col min="13319" max="13319" width="23.5" style="3" customWidth="1"/>
-    <col min="13320" max="13320" width="44.1640625" style="3" customWidth="1"/>
-    <col min="13321" max="13321" width="26.5" style="3" customWidth="1"/>
-    <col min="13322" max="13322" width="34.1640625" style="3" customWidth="1"/>
+    <col min="13316" max="13316" width="17.109375" style="3" customWidth="1"/>
+    <col min="13317" max="13317" width="13.77734375" style="3" customWidth="1"/>
+    <col min="13318" max="13318" width="11.109375" style="3" customWidth="1"/>
+    <col min="13319" max="13319" width="23.44140625" style="3" customWidth="1"/>
+    <col min="13320" max="13320" width="44.109375" style="3" customWidth="1"/>
+    <col min="13321" max="13321" width="26.44140625" style="3" customWidth="1"/>
+    <col min="13322" max="13322" width="34.109375" style="3" customWidth="1"/>
     <col min="13323" max="13323" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="13324" max="13568" width="8.83203125" style="3"/>
+    <col min="13324" max="13568" width="8.77734375" style="3"/>
     <col min="13569" max="13569" width="2.33203125" style="3" customWidth="1"/>
     <col min="13570" max="13570" width="57.6640625" style="3" customWidth="1"/>
     <col min="13571" max="13571" width="18.6640625" style="3" customWidth="1"/>
-    <col min="13572" max="13572" width="17.1640625" style="3" customWidth="1"/>
-    <col min="13573" max="13573" width="13.83203125" style="3" customWidth="1"/>
-    <col min="13574" max="13574" width="11.1640625" style="3" customWidth="1"/>
-    <col min="13575" max="13575" width="23.5" style="3" customWidth="1"/>
-    <col min="13576" max="13576" width="44.1640625" style="3" customWidth="1"/>
-    <col min="13577" max="13577" width="26.5" style="3" customWidth="1"/>
-    <col min="13578" max="13578" width="34.1640625" style="3" customWidth="1"/>
+    <col min="13572" max="13572" width="17.109375" style="3" customWidth="1"/>
+    <col min="13573" max="13573" width="13.77734375" style="3" customWidth="1"/>
+    <col min="13574" max="13574" width="11.109375" style="3" customWidth="1"/>
+    <col min="13575" max="13575" width="23.44140625" style="3" customWidth="1"/>
+    <col min="13576" max="13576" width="44.109375" style="3" customWidth="1"/>
+    <col min="13577" max="13577" width="26.44140625" style="3" customWidth="1"/>
+    <col min="13578" max="13578" width="34.109375" style="3" customWidth="1"/>
     <col min="13579" max="13579" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="13580" max="13824" width="8.83203125" style="3"/>
+    <col min="13580" max="13824" width="8.77734375" style="3"/>
     <col min="13825" max="13825" width="2.33203125" style="3" customWidth="1"/>
     <col min="13826" max="13826" width="57.6640625" style="3" customWidth="1"/>
     <col min="13827" max="13827" width="18.6640625" style="3" customWidth="1"/>
-    <col min="13828" max="13828" width="17.1640625" style="3" customWidth="1"/>
-    <col min="13829" max="13829" width="13.83203125" style="3" customWidth="1"/>
-    <col min="13830" max="13830" width="11.1640625" style="3" customWidth="1"/>
-    <col min="13831" max="13831" width="23.5" style="3" customWidth="1"/>
-    <col min="13832" max="13832" width="44.1640625" style="3" customWidth="1"/>
-    <col min="13833" max="13833" width="26.5" style="3" customWidth="1"/>
-    <col min="13834" max="13834" width="34.1640625" style="3" customWidth="1"/>
+    <col min="13828" max="13828" width="17.109375" style="3" customWidth="1"/>
+    <col min="13829" max="13829" width="13.77734375" style="3" customWidth="1"/>
+    <col min="13830" max="13830" width="11.109375" style="3" customWidth="1"/>
+    <col min="13831" max="13831" width="23.44140625" style="3" customWidth="1"/>
+    <col min="13832" max="13832" width="44.109375" style="3" customWidth="1"/>
+    <col min="13833" max="13833" width="26.44140625" style="3" customWidth="1"/>
+    <col min="13834" max="13834" width="34.109375" style="3" customWidth="1"/>
     <col min="13835" max="13835" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="13836" max="14080" width="8.83203125" style="3"/>
+    <col min="13836" max="14080" width="8.77734375" style="3"/>
     <col min="14081" max="14081" width="2.33203125" style="3" customWidth="1"/>
     <col min="14082" max="14082" width="57.6640625" style="3" customWidth="1"/>
     <col min="14083" max="14083" width="18.6640625" style="3" customWidth="1"/>
-    <col min="14084" max="14084" width="17.1640625" style="3" customWidth="1"/>
-    <col min="14085" max="14085" width="13.83203125" style="3" customWidth="1"/>
-    <col min="14086" max="14086" width="11.1640625" style="3" customWidth="1"/>
-    <col min="14087" max="14087" width="23.5" style="3" customWidth="1"/>
-    <col min="14088" max="14088" width="44.1640625" style="3" customWidth="1"/>
-    <col min="14089" max="14089" width="26.5" style="3" customWidth="1"/>
-    <col min="14090" max="14090" width="34.1640625" style="3" customWidth="1"/>
+    <col min="14084" max="14084" width="17.109375" style="3" customWidth="1"/>
+    <col min="14085" max="14085" width="13.77734375" style="3" customWidth="1"/>
+    <col min="14086" max="14086" width="11.109375" style="3" customWidth="1"/>
+    <col min="14087" max="14087" width="23.44140625" style="3" customWidth="1"/>
+    <col min="14088" max="14088" width="44.109375" style="3" customWidth="1"/>
+    <col min="14089" max="14089" width="26.44140625" style="3" customWidth="1"/>
+    <col min="14090" max="14090" width="34.109375" style="3" customWidth="1"/>
     <col min="14091" max="14091" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="14092" max="14336" width="8.83203125" style="3"/>
+    <col min="14092" max="14336" width="8.77734375" style="3"/>
     <col min="14337" max="14337" width="2.33203125" style="3" customWidth="1"/>
     <col min="14338" max="14338" width="57.6640625" style="3" customWidth="1"/>
     <col min="14339" max="14339" width="18.6640625" style="3" customWidth="1"/>
-    <col min="14340" max="14340" width="17.1640625" style="3" customWidth="1"/>
-    <col min="14341" max="14341" width="13.83203125" style="3" customWidth="1"/>
-    <col min="14342" max="14342" width="11.1640625" style="3" customWidth="1"/>
-    <col min="14343" max="14343" width="23.5" style="3" customWidth="1"/>
-    <col min="14344" max="14344" width="44.1640625" style="3" customWidth="1"/>
-    <col min="14345" max="14345" width="26.5" style="3" customWidth="1"/>
-    <col min="14346" max="14346" width="34.1640625" style="3" customWidth="1"/>
+    <col min="14340" max="14340" width="17.109375" style="3" customWidth="1"/>
+    <col min="14341" max="14341" width="13.77734375" style="3" customWidth="1"/>
+    <col min="14342" max="14342" width="11.109375" style="3" customWidth="1"/>
+    <col min="14343" max="14343" width="23.44140625" style="3" customWidth="1"/>
+    <col min="14344" max="14344" width="44.109375" style="3" customWidth="1"/>
+    <col min="14345" max="14345" width="26.44140625" style="3" customWidth="1"/>
+    <col min="14346" max="14346" width="34.109375" style="3" customWidth="1"/>
     <col min="14347" max="14347" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="14348" max="14592" width="8.83203125" style="3"/>
+    <col min="14348" max="14592" width="8.77734375" style="3"/>
     <col min="14593" max="14593" width="2.33203125" style="3" customWidth="1"/>
     <col min="14594" max="14594" width="57.6640625" style="3" customWidth="1"/>
     <col min="14595" max="14595" width="18.6640625" style="3" customWidth="1"/>
-    <col min="14596" max="14596" width="17.1640625" style="3" customWidth="1"/>
-    <col min="14597" max="14597" width="13.83203125" style="3" customWidth="1"/>
-    <col min="14598" max="14598" width="11.1640625" style="3" customWidth="1"/>
-    <col min="14599" max="14599" width="23.5" style="3" customWidth="1"/>
-    <col min="14600" max="14600" width="44.1640625" style="3" customWidth="1"/>
-    <col min="14601" max="14601" width="26.5" style="3" customWidth="1"/>
-    <col min="14602" max="14602" width="34.1640625" style="3" customWidth="1"/>
+    <col min="14596" max="14596" width="17.109375" style="3" customWidth="1"/>
+    <col min="14597" max="14597" width="13.77734375" style="3" customWidth="1"/>
+    <col min="14598" max="14598" width="11.109375" style="3" customWidth="1"/>
+    <col min="14599" max="14599" width="23.44140625" style="3" customWidth="1"/>
+    <col min="14600" max="14600" width="44.109375" style="3" customWidth="1"/>
+    <col min="14601" max="14601" width="26.44140625" style="3" customWidth="1"/>
+    <col min="14602" max="14602" width="34.109375" style="3" customWidth="1"/>
     <col min="14603" max="14603" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="14604" max="14848" width="8.83203125" style="3"/>
+    <col min="14604" max="14848" width="8.77734375" style="3"/>
     <col min="14849" max="14849" width="2.33203125" style="3" customWidth="1"/>
     <col min="14850" max="14850" width="57.6640625" style="3" customWidth="1"/>
     <col min="14851" max="14851" width="18.6640625" style="3" customWidth="1"/>
-    <col min="14852" max="14852" width="17.1640625" style="3" customWidth="1"/>
-    <col min="14853" max="14853" width="13.83203125" style="3" customWidth="1"/>
-    <col min="14854" max="14854" width="11.1640625" style="3" customWidth="1"/>
-    <col min="14855" max="14855" width="23.5" style="3" customWidth="1"/>
-    <col min="14856" max="14856" width="44.1640625" style="3" customWidth="1"/>
-    <col min="14857" max="14857" width="26.5" style="3" customWidth="1"/>
-    <col min="14858" max="14858" width="34.1640625" style="3" customWidth="1"/>
+    <col min="14852" max="14852" width="17.109375" style="3" customWidth="1"/>
+    <col min="14853" max="14853" width="13.77734375" style="3" customWidth="1"/>
+    <col min="14854" max="14854" width="11.109375" style="3" customWidth="1"/>
+    <col min="14855" max="14855" width="23.44140625" style="3" customWidth="1"/>
+    <col min="14856" max="14856" width="44.109375" style="3" customWidth="1"/>
+    <col min="14857" max="14857" width="26.44140625" style="3" customWidth="1"/>
+    <col min="14858" max="14858" width="34.109375" style="3" customWidth="1"/>
     <col min="14859" max="14859" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="14860" max="15104" width="8.83203125" style="3"/>
+    <col min="14860" max="15104" width="8.77734375" style="3"/>
     <col min="15105" max="15105" width="2.33203125" style="3" customWidth="1"/>
     <col min="15106" max="15106" width="57.6640625" style="3" customWidth="1"/>
     <col min="15107" max="15107" width="18.6640625" style="3" customWidth="1"/>
-    <col min="15108" max="15108" width="17.1640625" style="3" customWidth="1"/>
-    <col min="15109" max="15109" width="13.83203125" style="3" customWidth="1"/>
-    <col min="15110" max="15110" width="11.1640625" style="3" customWidth="1"/>
-    <col min="15111" max="15111" width="23.5" style="3" customWidth="1"/>
-    <col min="15112" max="15112" width="44.1640625" style="3" customWidth="1"/>
-    <col min="15113" max="15113" width="26.5" style="3" customWidth="1"/>
-    <col min="15114" max="15114" width="34.1640625" style="3" customWidth="1"/>
+    <col min="15108" max="15108" width="17.109375" style="3" customWidth="1"/>
+    <col min="15109" max="15109" width="13.77734375" style="3" customWidth="1"/>
+    <col min="15110" max="15110" width="11.109375" style="3" customWidth="1"/>
+    <col min="15111" max="15111" width="23.44140625" style="3" customWidth="1"/>
+    <col min="15112" max="15112" width="44.109375" style="3" customWidth="1"/>
+    <col min="15113" max="15113" width="26.44140625" style="3" customWidth="1"/>
+    <col min="15114" max="15114" width="34.109375" style="3" customWidth="1"/>
     <col min="15115" max="15115" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="15116" max="15360" width="8.83203125" style="3"/>
+    <col min="15116" max="15360" width="8.77734375" style="3"/>
     <col min="15361" max="15361" width="2.33203125" style="3" customWidth="1"/>
     <col min="15362" max="15362" width="57.6640625" style="3" customWidth="1"/>
     <col min="15363" max="15363" width="18.6640625" style="3" customWidth="1"/>
-    <col min="15364" max="15364" width="17.1640625" style="3" customWidth="1"/>
-    <col min="15365" max="15365" width="13.83203125" style="3" customWidth="1"/>
-    <col min="15366" max="15366" width="11.1640625" style="3" customWidth="1"/>
-    <col min="15367" max="15367" width="23.5" style="3" customWidth="1"/>
-    <col min="15368" max="15368" width="44.1640625" style="3" customWidth="1"/>
-    <col min="15369" max="15369" width="26.5" style="3" customWidth="1"/>
-    <col min="15370" max="15370" width="34.1640625" style="3" customWidth="1"/>
+    <col min="15364" max="15364" width="17.109375" style="3" customWidth="1"/>
+    <col min="15365" max="15365" width="13.77734375" style="3" customWidth="1"/>
+    <col min="15366" max="15366" width="11.109375" style="3" customWidth="1"/>
+    <col min="15367" max="15367" width="23.44140625" style="3" customWidth="1"/>
+    <col min="15368" max="15368" width="44.109375" style="3" customWidth="1"/>
+    <col min="15369" max="15369" width="26.44140625" style="3" customWidth="1"/>
+    <col min="15370" max="15370" width="34.109375" style="3" customWidth="1"/>
     <col min="15371" max="15371" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="15372" max="15616" width="8.83203125" style="3"/>
+    <col min="15372" max="15616" width="8.77734375" style="3"/>
     <col min="15617" max="15617" width="2.33203125" style="3" customWidth="1"/>
     <col min="15618" max="15618" width="57.6640625" style="3" customWidth="1"/>
     <col min="15619" max="15619" width="18.6640625" style="3" customWidth="1"/>
-    <col min="15620" max="15620" width="17.1640625" style="3" customWidth="1"/>
-    <col min="15621" max="15621" width="13.83203125" style="3" customWidth="1"/>
-    <col min="15622" max="15622" width="11.1640625" style="3" customWidth="1"/>
-    <col min="15623" max="15623" width="23.5" style="3" customWidth="1"/>
-    <col min="15624" max="15624" width="44.1640625" style="3" customWidth="1"/>
-    <col min="15625" max="15625" width="26.5" style="3" customWidth="1"/>
-    <col min="15626" max="15626" width="34.1640625" style="3" customWidth="1"/>
+    <col min="15620" max="15620" width="17.109375" style="3" customWidth="1"/>
+    <col min="15621" max="15621" width="13.77734375" style="3" customWidth="1"/>
+    <col min="15622" max="15622" width="11.109375" style="3" customWidth="1"/>
+    <col min="15623" max="15623" width="23.44140625" style="3" customWidth="1"/>
+    <col min="15624" max="15624" width="44.109375" style="3" customWidth="1"/>
+    <col min="15625" max="15625" width="26.44140625" style="3" customWidth="1"/>
+    <col min="15626" max="15626" width="34.109375" style="3" customWidth="1"/>
     <col min="15627" max="15627" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="15628" max="15872" width="8.83203125" style="3"/>
+    <col min="15628" max="15872" width="8.77734375" style="3"/>
     <col min="15873" max="15873" width="2.33203125" style="3" customWidth="1"/>
     <col min="15874" max="15874" width="57.6640625" style="3" customWidth="1"/>
     <col min="15875" max="15875" width="18.6640625" style="3" customWidth="1"/>
-    <col min="15876" max="15876" width="17.1640625" style="3" customWidth="1"/>
-    <col min="15877" max="15877" width="13.83203125" style="3" customWidth="1"/>
-    <col min="15878" max="15878" width="11.1640625" style="3" customWidth="1"/>
-    <col min="15879" max="15879" width="23.5" style="3" customWidth="1"/>
-    <col min="15880" max="15880" width="44.1640625" style="3" customWidth="1"/>
-    <col min="15881" max="15881" width="26.5" style="3" customWidth="1"/>
-    <col min="15882" max="15882" width="34.1640625" style="3" customWidth="1"/>
+    <col min="15876" max="15876" width="17.109375" style="3" customWidth="1"/>
+    <col min="15877" max="15877" width="13.77734375" style="3" customWidth="1"/>
+    <col min="15878" max="15878" width="11.109375" style="3" customWidth="1"/>
+    <col min="15879" max="15879" width="23.44140625" style="3" customWidth="1"/>
+    <col min="15880" max="15880" width="44.109375" style="3" customWidth="1"/>
+    <col min="15881" max="15881" width="26.44140625" style="3" customWidth="1"/>
+    <col min="15882" max="15882" width="34.109375" style="3" customWidth="1"/>
     <col min="15883" max="15883" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="15884" max="16128" width="8.83203125" style="3"/>
+    <col min="15884" max="16128" width="8.77734375" style="3"/>
     <col min="16129" max="16129" width="2.33203125" style="3" customWidth="1"/>
     <col min="16130" max="16130" width="57.6640625" style="3" customWidth="1"/>
     <col min="16131" max="16131" width="18.6640625" style="3" customWidth="1"/>
-    <col min="16132" max="16132" width="17.1640625" style="3" customWidth="1"/>
-    <col min="16133" max="16133" width="13.83203125" style="3" customWidth="1"/>
-    <col min="16134" max="16134" width="11.1640625" style="3" customWidth="1"/>
-    <col min="16135" max="16135" width="23.5" style="3" customWidth="1"/>
-    <col min="16136" max="16136" width="44.1640625" style="3" customWidth="1"/>
-    <col min="16137" max="16137" width="26.5" style="3" customWidth="1"/>
-    <col min="16138" max="16138" width="34.1640625" style="3" customWidth="1"/>
+    <col min="16132" max="16132" width="17.109375" style="3" customWidth="1"/>
+    <col min="16133" max="16133" width="13.77734375" style="3" customWidth="1"/>
+    <col min="16134" max="16134" width="11.109375" style="3" customWidth="1"/>
+    <col min="16135" max="16135" width="23.44140625" style="3" customWidth="1"/>
+    <col min="16136" max="16136" width="44.109375" style="3" customWidth="1"/>
+    <col min="16137" max="16137" width="26.44140625" style="3" customWidth="1"/>
+    <col min="16138" max="16138" width="34.109375" style="3" customWidth="1"/>
     <col min="16139" max="16139" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="16140" max="16384" width="8.83203125" style="3"/>
+    <col min="16140" max="16384" width="8.77734375" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="45">
+    <row r="1" spans="1:13" ht="44.4">
       <c r="A1" s="1"/>
       <c r="B1" s="19" t="s">
         <v>0</v>
@@ -3537,254 +3588,254 @@
       <c r="L1" s="2"/>
       <c r="M1" s="2"/>
     </row>
-    <row r="2" spans="1:13" ht="83" customHeight="1">
+    <row r="2" spans="1:13" ht="82.95" customHeight="1">
       <c r="A2" s="4"/>
       <c r="B2" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="172">
+      <c r="C2" s="186">
         <v>46020</v>
       </c>
-      <c r="D2" s="173"/>
-      <c r="E2" s="174"/>
-      <c r="F2" s="175" t="s">
+      <c r="D2" s="187"/>
+      <c r="E2" s="188"/>
+      <c r="F2" s="189" t="s">
         <v>29</v>
       </c>
-      <c r="G2" s="176"/>
-      <c r="H2" s="177" t="s">
+      <c r="G2" s="190"/>
+      <c r="H2" s="191" t="s">
         <v>60</v>
       </c>
-      <c r="I2" s="178"/>
-      <c r="J2" s="178"/>
-      <c r="K2" s="179"/>
+      <c r="I2" s="192"/>
+      <c r="J2" s="192"/>
+      <c r="K2" s="193"/>
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
     </row>
-    <row r="3" spans="1:13" ht="74" customHeight="1">
+    <row r="3" spans="1:13" ht="73.95" customHeight="1">
       <c r="A3" s="4"/>
       <c r="B3" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="C3" s="172" t="s">
+      <c r="C3" s="186" t="s">
         <v>61</v>
       </c>
-      <c r="D3" s="173"/>
-      <c r="E3" s="174"/>
-      <c r="F3" s="180"/>
-      <c r="G3" s="181"/>
-      <c r="H3" s="200" t="s">
+      <c r="D3" s="187"/>
+      <c r="E3" s="188"/>
+      <c r="F3" s="194"/>
+      <c r="G3" s="195"/>
+      <c r="H3" s="214" t="s">
         <v>39</v>
       </c>
-      <c r="I3" s="201"/>
+      <c r="I3" s="215"/>
       <c r="J3" s="59"/>
       <c r="K3" s="60"/>
       <c r="L3" s="2"/>
       <c r="M3" s="2"/>
     </row>
-    <row r="4" spans="1:13" ht="74" customHeight="1">
+    <row r="4" spans="1:13" ht="73.95" customHeight="1">
       <c r="A4" s="4"/>
       <c r="B4" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="186" t="s">
+      <c r="C4" s="200" t="s">
         <v>68</v>
       </c>
-      <c r="D4" s="187"/>
-      <c r="E4" s="188"/>
-      <c r="F4" s="182"/>
-      <c r="G4" s="183"/>
-      <c r="H4" s="168"/>
-      <c r="I4" s="169"/>
-      <c r="J4" s="166"/>
-      <c r="K4" s="167"/>
+      <c r="D4" s="201"/>
+      <c r="E4" s="202"/>
+      <c r="F4" s="196"/>
+      <c r="G4" s="197"/>
+      <c r="H4" s="166"/>
+      <c r="I4" s="167"/>
+      <c r="J4" s="216"/>
+      <c r="K4" s="217"/>
       <c r="L4" s="2"/>
       <c r="M4" s="2"/>
     </row>
-    <row r="5" spans="1:13" ht="74" customHeight="1">
+    <row r="5" spans="1:13" ht="73.95" customHeight="1">
       <c r="A5" s="4"/>
       <c r="B5" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="189">
+      <c r="C5" s="203">
         <v>51311172</v>
       </c>
-      <c r="D5" s="190"/>
-      <c r="E5" s="191"/>
-      <c r="F5" s="182"/>
-      <c r="G5" s="183"/>
-      <c r="H5" s="168"/>
-      <c r="I5" s="169"/>
-      <c r="J5" s="166"/>
-      <c r="K5" s="167"/>
+      <c r="D5" s="204"/>
+      <c r="E5" s="205"/>
+      <c r="F5" s="196"/>
+      <c r="G5" s="197"/>
+      <c r="H5" s="166"/>
+      <c r="I5" s="167"/>
+      <c r="J5" s="216"/>
+      <c r="K5" s="217"/>
       <c r="L5" s="2"/>
       <c r="M5" s="2"/>
     </row>
-    <row r="6" spans="1:13" ht="74" customHeight="1">
+    <row r="6" spans="1:13" ht="73.95" customHeight="1">
       <c r="A6" s="4"/>
       <c r="B6" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="189" t="s">
+      <c r="C6" s="203" t="s">
         <v>69</v>
       </c>
-      <c r="D6" s="190"/>
-      <c r="E6" s="191"/>
-      <c r="F6" s="182"/>
-      <c r="G6" s="183"/>
-      <c r="H6" s="168"/>
-      <c r="I6" s="169"/>
-      <c r="J6" s="166"/>
-      <c r="K6" s="167"/>
+      <c r="D6" s="204"/>
+      <c r="E6" s="205"/>
+      <c r="F6" s="196"/>
+      <c r="G6" s="197"/>
+      <c r="H6" s="166"/>
+      <c r="I6" s="167"/>
+      <c r="J6" s="216"/>
+      <c r="K6" s="217"/>
       <c r="L6" s="2"/>
       <c r="M6" s="2"/>
     </row>
-    <row r="7" spans="1:13" ht="74" customHeight="1">
+    <row r="7" spans="1:13" ht="73.95" customHeight="1">
       <c r="A7" s="4"/>
       <c r="B7" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="C7" s="189" t="s">
+      <c r="C7" s="203" t="s">
         <v>53</v>
       </c>
-      <c r="D7" s="190"/>
-      <c r="E7" s="191"/>
-      <c r="F7" s="182"/>
-      <c r="G7" s="183"/>
-      <c r="H7" s="168"/>
-      <c r="I7" s="169"/>
-      <c r="J7" s="166"/>
-      <c r="K7" s="167"/>
+      <c r="D7" s="204"/>
+      <c r="E7" s="205"/>
+      <c r="F7" s="196"/>
+      <c r="G7" s="197"/>
+      <c r="H7" s="166"/>
+      <c r="I7" s="167"/>
+      <c r="J7" s="216"/>
+      <c r="K7" s="217"/>
       <c r="L7" s="2"/>
       <c r="M7" s="2"/>
     </row>
-    <row r="8" spans="1:13" ht="74" customHeight="1">
+    <row r="8" spans="1:13" ht="73.95" customHeight="1">
       <c r="A8" s="4"/>
       <c r="B8" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="192" t="s">
+      <c r="C8" s="206" t="s">
         <v>71</v>
       </c>
-      <c r="D8" s="173"/>
-      <c r="E8" s="193"/>
-      <c r="F8" s="182"/>
-      <c r="G8" s="183"/>
+      <c r="D8" s="187"/>
+      <c r="E8" s="207"/>
+      <c r="F8" s="196"/>
+      <c r="G8" s="197"/>
       <c r="H8" s="72"/>
       <c r="I8" s="73"/>
-      <c r="J8" s="166"/>
-      <c r="K8" s="167"/>
+      <c r="J8" s="216"/>
+      <c r="K8" s="217"/>
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
     </row>
-    <row r="9" spans="1:13" ht="74" customHeight="1">
+    <row r="9" spans="1:13" ht="73.95" customHeight="1">
       <c r="A9" s="4"/>
       <c r="B9" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="C9" s="197"/>
-      <c r="D9" s="198"/>
-      <c r="E9" s="199"/>
-      <c r="F9" s="182"/>
-      <c r="G9" s="183"/>
+      <c r="C9" s="211"/>
+      <c r="D9" s="212"/>
+      <c r="E9" s="213"/>
+      <c r="F9" s="196"/>
+      <c r="G9" s="197"/>
       <c r="H9" s="72"/>
       <c r="I9" s="73"/>
-      <c r="J9" s="166"/>
-      <c r="K9" s="167"/>
+      <c r="J9" s="216"/>
+      <c r="K9" s="217"/>
       <c r="L9" s="2"/>
       <c r="M9" s="2"/>
     </row>
-    <row r="10" spans="1:13" ht="74" customHeight="1">
+    <row r="10" spans="1:13" ht="73.95" customHeight="1">
       <c r="A10" s="4"/>
       <c r="B10" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="C10" s="194"/>
-      <c r="D10" s="195"/>
-      <c r="E10" s="196"/>
-      <c r="F10" s="182"/>
-      <c r="G10" s="183"/>
+      <c r="C10" s="208"/>
+      <c r="D10" s="209"/>
+      <c r="E10" s="210"/>
+      <c r="F10" s="196"/>
+      <c r="G10" s="197"/>
       <c r="H10" s="72"/>
       <c r="I10" s="73"/>
-      <c r="J10" s="166"/>
-      <c r="K10" s="167"/>
+      <c r="J10" s="216"/>
+      <c r="K10" s="217"/>
       <c r="L10" s="2"/>
       <c r="M10" s="2"/>
     </row>
-    <row r="11" spans="1:13" ht="74" customHeight="1">
+    <row r="11" spans="1:13" ht="73.95" customHeight="1">
       <c r="A11" s="4"/>
       <c r="B11" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="C11" s="202"/>
-      <c r="D11" s="203"/>
-      <c r="E11" s="204"/>
-      <c r="F11" s="182"/>
-      <c r="G11" s="183"/>
-      <c r="H11" s="168"/>
-      <c r="I11" s="169"/>
-      <c r="J11" s="170"/>
-      <c r="K11" s="171"/>
+      <c r="C11" s="159"/>
+      <c r="D11" s="160"/>
+      <c r="E11" s="161"/>
+      <c r="F11" s="196"/>
+      <c r="G11" s="197"/>
+      <c r="H11" s="166"/>
+      <c r="I11" s="167"/>
+      <c r="J11" s="171"/>
+      <c r="K11" s="172"/>
       <c r="L11" s="2"/>
       <c r="M11" s="2"/>
     </row>
-    <row r="12" spans="1:13" ht="74" customHeight="1">
+    <row r="12" spans="1:13" ht="73.95" customHeight="1">
       <c r="A12" s="4"/>
       <c r="B12" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="226" t="s">
+      <c r="C12" s="156" t="s">
         <v>43</v>
       </c>
-      <c r="D12" s="227"/>
-      <c r="E12" s="228"/>
-      <c r="F12" s="182"/>
-      <c r="G12" s="183"/>
-      <c r="H12" s="168"/>
-      <c r="I12" s="169"/>
-      <c r="J12" s="170"/>
-      <c r="K12" s="171"/>
+      <c r="D12" s="157"/>
+      <c r="E12" s="158"/>
+      <c r="F12" s="196"/>
+      <c r="G12" s="197"/>
+      <c r="H12" s="166"/>
+      <c r="I12" s="167"/>
+      <c r="J12" s="171"/>
+      <c r="K12" s="172"/>
       <c r="L12" s="2"/>
       <c r="M12" s="2"/>
     </row>
-    <row r="13" spans="1:13" ht="74" customHeight="1">
+    <row r="13" spans="1:13" ht="73.95" customHeight="1">
       <c r="A13" s="4"/>
       <c r="B13" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="202"/>
-      <c r="D13" s="203"/>
-      <c r="E13" s="204"/>
-      <c r="F13" s="184"/>
-      <c r="G13" s="185"/>
-      <c r="H13" s="168"/>
-      <c r="I13" s="169"/>
-      <c r="J13" s="170"/>
-      <c r="K13" s="171"/>
+      <c r="C13" s="159"/>
+      <c r="D13" s="160"/>
+      <c r="E13" s="161"/>
+      <c r="F13" s="198"/>
+      <c r="G13" s="199"/>
+      <c r="H13" s="166"/>
+      <c r="I13" s="167"/>
+      <c r="J13" s="171"/>
+      <c r="K13" s="172"/>
       <c r="L13" s="2"/>
       <c r="M13" s="2"/>
     </row>
-    <row r="14" spans="1:13" ht="74" customHeight="1">
+    <row r="14" spans="1:13" ht="73.95" customHeight="1">
       <c r="A14" s="4"/>
       <c r="B14" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="C14" s="229" t="s">
+      <c r="C14" s="162" t="s">
         <v>67</v>
       </c>
-      <c r="D14" s="229"/>
-      <c r="E14" s="230"/>
-      <c r="F14" s="231" t="s">
+      <c r="D14" s="162"/>
+      <c r="E14" s="163"/>
+      <c r="F14" s="164" t="s">
         <v>70</v>
       </c>
-      <c r="G14" s="231"/>
-      <c r="H14" s="231"/>
-      <c r="I14" s="231"/>
+      <c r="G14" s="164"/>
+      <c r="H14" s="164"/>
+      <c r="I14" s="164"/>
       <c r="J14" s="26"/>
       <c r="K14" s="27"/>
       <c r="L14" s="2"/>
       <c r="M14" s="2"/>
     </row>
-    <row r="15" spans="1:13" ht="74" customHeight="1" thickBot="1">
+    <row r="15" spans="1:13" ht="73.95" customHeight="1" thickBot="1">
       <c r="A15" s="4"/>
       <c r="B15" s="76" t="s">
         <v>31</v>
@@ -3798,11 +3849,11 @@
       <c r="E15" s="79">
         <v>1</v>
       </c>
-      <c r="F15" s="232"/>
-      <c r="G15" s="232"/>
-      <c r="H15" s="232"/>
-      <c r="I15" s="232"/>
-      <c r="J15" s="218" t="s">
+      <c r="F15" s="165"/>
+      <c r="G15" s="165"/>
+      <c r="H15" s="165"/>
+      <c r="I15" s="165"/>
+      <c r="J15" s="173" t="s">
         <v>10</v>
       </c>
       <c r="K15" s="52" t="s">
@@ -3811,7 +3862,7 @@
       <c r="L15" s="2"/>
       <c r="M15" s="2"/>
     </row>
-    <row r="16" spans="1:13" ht="74" customHeight="1">
+    <row r="16" spans="1:13" ht="73.95" customHeight="1">
       <c r="A16" s="11"/>
       <c r="B16" s="32" t="s">
         <v>12</v>
@@ -3831,35 +3882,35 @@
       <c r="G16" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="H16" s="220" t="s">
+      <c r="H16" s="175" t="s">
         <v>17</v>
       </c>
-      <c r="I16" s="220"/>
-      <c r="J16" s="219"/>
+      <c r="I16" s="175"/>
+      <c r="J16" s="174"/>
       <c r="K16" s="28"/>
       <c r="L16" s="5"/>
       <c r="M16" s="5"/>
     </row>
-    <row r="17" spans="1:13" ht="98" customHeight="1">
+    <row r="17" spans="1:13" ht="97.95" customHeight="1">
       <c r="A17" s="6"/>
       <c r="B17" s="123" t="s">
         <v>42</v>
       </c>
-      <c r="C17" s="221" t="s">
+      <c r="C17" s="226" t="s">
         <v>56</v>
       </c>
-      <c r="D17" s="222"/>
-      <c r="E17" s="222"/>
-      <c r="F17" s="222"/>
-      <c r="G17" s="222"/>
-      <c r="H17" s="222"/>
-      <c r="I17" s="223"/>
+      <c r="D17" s="227"/>
+      <c r="E17" s="227"/>
+      <c r="F17" s="227"/>
+      <c r="G17" s="227"/>
+      <c r="H17" s="227"/>
+      <c r="I17" s="228"/>
       <c r="J17" s="29"/>
       <c r="K17" s="22"/>
       <c r="L17" s="5"/>
       <c r="M17" s="5"/>
     </row>
-    <row r="18" spans="1:13" ht="71" customHeight="1">
+    <row r="18" spans="1:13" ht="70.95" customHeight="1">
       <c r="A18" s="6"/>
       <c r="B18" s="99" t="s">
         <v>49</v>
@@ -3873,16 +3924,16 @@
       <c r="G18" s="34" t="s">
         <v>32</v>
       </c>
-      <c r="H18" s="155" t="s">
+      <c r="H18" s="218" t="s">
         <v>38</v>
       </c>
-      <c r="I18" s="156"/>
+      <c r="I18" s="219"/>
       <c r="J18" s="30"/>
       <c r="K18" s="44"/>
       <c r="L18" s="5"/>
       <c r="M18" s="5"/>
     </row>
-    <row r="19" spans="1:13" ht="85" customHeight="1">
+    <row r="19" spans="1:13" ht="85.05" customHeight="1">
       <c r="A19" s="6"/>
       <c r="B19" s="68" t="s">
         <v>40</v>
@@ -3891,15 +3942,15 @@
       <c r="D19" s="69"/>
       <c r="E19" s="70"/>
       <c r="F19" s="71"/>
-      <c r="G19" s="236"/>
-      <c r="H19" s="237"/>
-      <c r="I19" s="237"/>
+      <c r="G19" s="155"/>
+      <c r="H19" s="224"/>
+      <c r="I19" s="225"/>
       <c r="J19" s="30"/>
       <c r="K19" s="30"/>
       <c r="L19" s="5"/>
       <c r="M19" s="5"/>
     </row>
-    <row r="20" spans="1:13" ht="71" customHeight="1">
+    <row r="20" spans="1:13" ht="70.95" customHeight="1">
       <c r="A20" s="6"/>
       <c r="B20" s="138"/>
       <c r="C20" s="139"/>
@@ -3914,7 +3965,7 @@
       <c r="L20" s="5"/>
       <c r="M20" s="5"/>
     </row>
-    <row r="21" spans="1:13" ht="71" customHeight="1">
+    <row r="21" spans="1:13" ht="70.95" customHeight="1">
       <c r="A21" s="6"/>
       <c r="B21" s="144" t="s">
         <v>65</v>
@@ -3928,16 +3979,16 @@
       <c r="G21" s="145" t="s">
         <v>22</v>
       </c>
-      <c r="H21" s="159" t="s">
+      <c r="H21" s="220" t="s">
         <v>66</v>
       </c>
-      <c r="I21" s="159"/>
+      <c r="I21" s="221"/>
       <c r="J21" s="146"/>
       <c r="K21" s="147"/>
       <c r="L21" s="5"/>
       <c r="M21" s="5"/>
     </row>
-    <row r="22" spans="1:13" ht="71" customHeight="1">
+    <row r="22" spans="1:13" ht="70.95" customHeight="1">
       <c r="A22" s="6"/>
       <c r="B22" s="148" t="s">
         <v>40</v>
@@ -3949,14 +4000,14 @@
       <c r="E22" s="145"/>
       <c r="F22" s="145"/>
       <c r="G22" s="145"/>
-      <c r="H22" s="159"/>
-      <c r="I22" s="159"/>
+      <c r="H22" s="220"/>
+      <c r="I22" s="249"/>
       <c r="J22" s="146"/>
       <c r="K22" s="147"/>
       <c r="L22" s="5"/>
       <c r="M22" s="5"/>
     </row>
-    <row r="23" spans="1:13" ht="71" customHeight="1">
+    <row r="23" spans="1:13" ht="70.95" customHeight="1">
       <c r="A23" s="6"/>
       <c r="B23" s="150"/>
       <c r="C23" s="151"/>
@@ -3971,7 +4022,7 @@
       <c r="L23" s="5"/>
       <c r="M23" s="5"/>
     </row>
-    <row r="24" spans="1:13" ht="71" customHeight="1">
+    <row r="24" spans="1:13" ht="70.95" customHeight="1">
       <c r="A24" s="6"/>
       <c r="B24" s="124" t="s">
         <v>41</v>
@@ -3985,16 +4036,16 @@
       <c r="G24" s="44" t="s">
         <v>22</v>
       </c>
-      <c r="H24" s="157" t="s">
+      <c r="H24" s="220" t="s">
         <v>57</v>
       </c>
-      <c r="I24" s="157"/>
+      <c r="I24" s="221"/>
       <c r="J24" s="74"/>
       <c r="K24" s="126"/>
       <c r="L24" s="5"/>
       <c r="M24" s="5"/>
     </row>
-    <row r="25" spans="1:13" ht="71" customHeight="1">
+    <row r="25" spans="1:13" ht="70.95" customHeight="1">
       <c r="A25" s="6"/>
       <c r="B25" s="32"/>
       <c r="C25" s="33"/>
@@ -4006,16 +4057,16 @@
       <c r="G25" s="44" t="s">
         <v>22</v>
       </c>
-      <c r="H25" s="158" t="s">
+      <c r="H25" s="222" t="s">
         <v>62</v>
       </c>
-      <c r="I25" s="158"/>
+      <c r="I25" s="247"/>
       <c r="J25" s="30"/>
       <c r="K25" s="127"/>
       <c r="L25" s="5"/>
       <c r="M25" s="5"/>
     </row>
-    <row r="26" spans="1:13" ht="71" customHeight="1">
+    <row r="26" spans="1:13" ht="70.95" customHeight="1">
       <c r="A26" s="6"/>
       <c r="B26" s="87" t="s">
         <v>18</v>
@@ -4029,14 +4080,14 @@
       <c r="E26" s="88"/>
       <c r="F26" s="89"/>
       <c r="G26" s="84"/>
-      <c r="H26" s="162"/>
-      <c r="I26" s="163"/>
+      <c r="H26" s="239"/>
+      <c r="I26" s="240"/>
       <c r="J26" s="85"/>
       <c r="K26" s="90"/>
       <c r="L26" s="5"/>
       <c r="M26" s="5"/>
     </row>
-    <row r="27" spans="1:13" ht="71" customHeight="1">
+    <row r="27" spans="1:13" ht="70.95" customHeight="1">
       <c r="A27" s="6" t="s">
         <v>59</v>
       </c>
@@ -4050,14 +4101,14 @@
       <c r="E27" s="88"/>
       <c r="F27" s="83"/>
       <c r="G27" s="83"/>
-      <c r="H27" s="164"/>
-      <c r="I27" s="165"/>
+      <c r="H27" s="237"/>
+      <c r="I27" s="246"/>
       <c r="J27" s="83"/>
       <c r="K27" s="83"/>
       <c r="L27" s="5"/>
       <c r="M27" s="5"/>
     </row>
-    <row r="28" spans="1:13" ht="71" customHeight="1">
+    <row r="28" spans="1:13" ht="70.95" customHeight="1">
       <c r="A28" s="6"/>
       <c r="B28" s="128"/>
       <c r="C28" s="129"/>
@@ -4065,14 +4116,14 @@
       <c r="E28" s="129"/>
       <c r="F28" s="129"/>
       <c r="G28" s="129"/>
-      <c r="H28" s="234"/>
-      <c r="I28" s="235"/>
+      <c r="H28" s="244"/>
+      <c r="I28" s="245"/>
       <c r="J28" s="130"/>
       <c r="K28" s="130"/>
       <c r="L28" s="5"/>
       <c r="M28" s="5"/>
     </row>
-    <row r="29" spans="1:13" ht="71" customHeight="1">
+    <row r="29" spans="1:13" ht="70.95" customHeight="1">
       <c r="A29" s="6"/>
       <c r="B29" s="124" t="s">
         <v>41</v>
@@ -4086,16 +4137,16 @@
       <c r="G29" s="44" t="s">
         <v>22</v>
       </c>
-      <c r="H29" s="157" t="s">
+      <c r="H29" s="220" t="s">
         <v>57</v>
       </c>
-      <c r="I29" s="157"/>
+      <c r="I29" s="221"/>
       <c r="J29" s="74"/>
       <c r="K29" s="126"/>
       <c r="L29" s="5"/>
       <c r="M29" s="5"/>
     </row>
-    <row r="30" spans="1:13" ht="71" customHeight="1">
+    <row r="30" spans="1:13" ht="70.95" customHeight="1">
       <c r="A30" s="6"/>
       <c r="B30" s="32"/>
       <c r="C30" s="33"/>
@@ -4107,16 +4158,16 @@
       <c r="G30" s="44" t="s">
         <v>22</v>
       </c>
-      <c r="H30" s="158" t="s">
+      <c r="H30" s="222" t="s">
         <v>58</v>
       </c>
-      <c r="I30" s="158"/>
+      <c r="I30" s="223"/>
       <c r="J30" s="30"/>
       <c r="K30" s="127"/>
       <c r="L30" s="5"/>
       <c r="M30" s="5"/>
     </row>
-    <row r="31" spans="1:13" ht="71" customHeight="1">
+    <row r="31" spans="1:13" ht="70.95" customHeight="1">
       <c r="A31" s="6"/>
       <c r="B31" s="61" t="s">
         <v>46</v>
@@ -4130,14 +4181,14 @@
       <c r="E31" s="62"/>
       <c r="F31" s="65"/>
       <c r="G31" s="66"/>
-      <c r="H31" s="233"/>
-      <c r="I31" s="233"/>
+      <c r="H31" s="222"/>
+      <c r="I31" s="223"/>
       <c r="J31" s="65"/>
       <c r="K31" s="67"/>
       <c r="L31" s="5"/>
       <c r="M31" s="5"/>
     </row>
-    <row r="32" spans="1:13" ht="74" customHeight="1">
+    <row r="32" spans="1:13" ht="73.95" customHeight="1">
       <c r="A32" s="7"/>
       <c r="B32" s="91"/>
       <c r="C32" s="92"/>
@@ -4152,7 +4203,7 @@
       <c r="L32" s="2"/>
       <c r="M32" s="8"/>
     </row>
-    <row r="33" spans="1:13" ht="74" customHeight="1">
+    <row r="33" spans="1:13" ht="73.95" customHeight="1">
       <c r="A33" s="7"/>
       <c r="B33" s="137" t="s">
         <v>63</v>
@@ -4164,16 +4215,16 @@
       <c r="E33" s="75"/>
       <c r="F33" s="75"/>
       <c r="G33" s="44"/>
-      <c r="H33" s="157" t="s">
+      <c r="H33" s="220" t="s">
         <v>72</v>
       </c>
-      <c r="I33" s="157"/>
+      <c r="I33" s="249"/>
       <c r="J33" s="74"/>
       <c r="K33" s="126"/>
       <c r="L33" s="2"/>
       <c r="M33" s="8"/>
     </row>
-    <row r="34" spans="1:13" ht="74" customHeight="1">
+    <row r="34" spans="1:13" ht="73.95" customHeight="1">
       <c r="A34" s="7"/>
       <c r="B34" s="32" t="s">
         <v>64</v>
@@ -4185,14 +4236,14 @@
       <c r="E34" s="33"/>
       <c r="F34" s="75"/>
       <c r="G34" s="44"/>
-      <c r="H34" s="158"/>
-      <c r="I34" s="158"/>
+      <c r="H34" s="222"/>
+      <c r="I34" s="247"/>
       <c r="J34" s="30"/>
       <c r="K34" s="127"/>
       <c r="L34" s="2"/>
       <c r="M34" s="8"/>
     </row>
-    <row r="35" spans="1:13" ht="74" customHeight="1">
+    <row r="35" spans="1:13" ht="73.95" customHeight="1">
       <c r="A35" s="7"/>
       <c r="B35" s="131"/>
       <c r="C35" s="132"/>
@@ -4207,7 +4258,7 @@
       <c r="L35" s="2"/>
       <c r="M35" s="8"/>
     </row>
-    <row r="36" spans="1:13" ht="74" customHeight="1">
+    <row r="36" spans="1:13" ht="73.95" customHeight="1">
       <c r="A36" s="7"/>
       <c r="B36" s="96" t="s">
         <v>44</v>
@@ -4221,16 +4272,16 @@
       <c r="G36" s="81" t="s">
         <v>32</v>
       </c>
-      <c r="H36" s="161" t="s">
+      <c r="H36" s="237" t="s">
         <v>21</v>
       </c>
-      <c r="I36" s="161"/>
+      <c r="I36" s="238"/>
       <c r="J36" s="83"/>
       <c r="K36" s="83"/>
       <c r="L36" s="2"/>
       <c r="M36" s="8"/>
     </row>
-    <row r="37" spans="1:13" ht="74" customHeight="1">
+    <row r="37" spans="1:13" ht="73.95" customHeight="1">
       <c r="A37" s="7"/>
       <c r="B37" s="87" t="s">
         <v>18</v>
@@ -4246,16 +4297,16 @@
       <c r="G37" s="83" t="s">
         <v>22</v>
       </c>
-      <c r="H37" s="164" t="s">
+      <c r="H37" s="237" t="s">
         <v>48</v>
       </c>
-      <c r="I37" s="165"/>
+      <c r="I37" s="238"/>
       <c r="J37" s="83"/>
       <c r="K37" s="83"/>
       <c r="L37" s="2"/>
       <c r="M37" s="8"/>
     </row>
-    <row r="38" spans="1:13" ht="74" customHeight="1">
+    <row r="38" spans="1:13" ht="73.95" customHeight="1">
       <c r="A38" s="7"/>
       <c r="B38" s="91"/>
       <c r="C38" s="92"/>
@@ -4270,7 +4321,7 @@
       <c r="L38" s="2"/>
       <c r="M38" s="8"/>
     </row>
-    <row r="39" spans="1:13" ht="74" customHeight="1">
+    <row r="39" spans="1:13" ht="73.95" customHeight="1">
       <c r="A39" s="7"/>
       <c r="B39" s="97" t="s">
         <v>20</v>
@@ -4286,16 +4337,16 @@
       <c r="G39" s="84" t="s">
         <v>32</v>
       </c>
-      <c r="H39" s="161" t="s">
+      <c r="H39" s="237" t="s">
         <v>37</v>
       </c>
-      <c r="I39" s="161"/>
+      <c r="I39" s="241"/>
       <c r="J39" s="85"/>
       <c r="K39" s="86"/>
       <c r="L39" s="2"/>
       <c r="M39" s="8"/>
     </row>
-    <row r="40" spans="1:13" ht="74" customHeight="1">
+    <row r="40" spans="1:13" ht="73.95" customHeight="1">
       <c r="A40" s="7"/>
       <c r="B40" s="87" t="s">
         <v>18</v>
@@ -4309,14 +4360,14 @@
       <c r="E40" s="88"/>
       <c r="F40" s="89"/>
       <c r="G40" s="84"/>
-      <c r="H40" s="162"/>
-      <c r="I40" s="163"/>
+      <c r="H40" s="239"/>
+      <c r="I40" s="240"/>
       <c r="J40" s="85"/>
       <c r="K40" s="90"/>
       <c r="L40" s="2"/>
       <c r="M40" s="8"/>
     </row>
-    <row r="41" spans="1:13" ht="74" customHeight="1">
+    <row r="41" spans="1:13" ht="73.95" customHeight="1">
       <c r="A41" s="7"/>
       <c r="B41" s="106"/>
       <c r="C41" s="107"/>
@@ -4331,7 +4382,7 @@
       <c r="L41" s="2"/>
       <c r="M41" s="8"/>
     </row>
-    <row r="42" spans="1:13" ht="74" customHeight="1">
+    <row r="42" spans="1:13" ht="73.95" customHeight="1">
       <c r="A42" s="7"/>
       <c r="B42" s="61" t="s">
         <v>45</v>
@@ -4345,16 +4396,16 @@
       <c r="G42" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="H42" s="160" t="s">
+      <c r="H42" s="242" t="s">
         <v>37</v>
       </c>
-      <c r="I42" s="160"/>
+      <c r="I42" s="248"/>
       <c r="J42" s="63"/>
       <c r="K42" s="63"/>
       <c r="L42" s="2"/>
       <c r="M42" s="8"/>
     </row>
-    <row r="43" spans="1:13" ht="74" customHeight="1">
+    <row r="43" spans="1:13" ht="73.95" customHeight="1">
       <c r="A43" s="7"/>
       <c r="B43" s="61" t="s">
         <v>46</v>
@@ -4370,16 +4421,16 @@
       <c r="G43" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="H43" s="160" t="s">
+      <c r="H43" s="242" t="s">
         <v>47</v>
       </c>
-      <c r="I43" s="160"/>
+      <c r="I43" s="243"/>
       <c r="J43" s="63"/>
       <c r="K43" s="63"/>
       <c r="L43" s="2"/>
       <c r="M43" s="8"/>
     </row>
-    <row r="44" spans="1:13" ht="74" customHeight="1">
+    <row r="44" spans="1:13" ht="73.95" customHeight="1">
       <c r="A44" s="7"/>
       <c r="B44" s="35"/>
       <c r="C44" s="36"/>
@@ -4387,14 +4438,14 @@
       <c r="E44" s="36"/>
       <c r="F44" s="31"/>
       <c r="G44" s="31"/>
-      <c r="H44" s="207"/>
-      <c r="I44" s="208"/>
+      <c r="H44" s="235"/>
+      <c r="I44" s="236"/>
       <c r="J44" s="31"/>
       <c r="K44" s="37"/>
       <c r="L44" s="2"/>
       <c r="M44" s="8"/>
     </row>
-    <row r="45" spans="1:13" ht="74" customHeight="1">
+    <row r="45" spans="1:13" ht="73.95" customHeight="1">
       <c r="A45" s="7"/>
       <c r="B45" s="98" t="s">
         <v>23</v>
@@ -4408,16 +4459,16 @@
       <c r="G45" s="55" t="s">
         <v>22</v>
       </c>
-      <c r="H45" s="211" t="s">
+      <c r="H45" s="231" t="s">
         <v>35</v>
       </c>
-      <c r="I45" s="211"/>
+      <c r="I45" s="232"/>
       <c r="J45" s="55"/>
       <c r="K45" s="55"/>
       <c r="L45" s="2"/>
       <c r="M45" s="8"/>
     </row>
-    <row r="46" spans="1:13" ht="74" customHeight="1">
+    <row r="46" spans="1:13" ht="73.95" customHeight="1">
       <c r="A46" s="7"/>
       <c r="B46" s="53"/>
       <c r="C46" s="54"/>
@@ -4427,16 +4478,16 @@
       <c r="G46" s="55" t="s">
         <v>22</v>
       </c>
-      <c r="H46" s="210" t="s">
+      <c r="H46" s="233" t="s">
         <v>36</v>
       </c>
-      <c r="I46" s="210"/>
+      <c r="I46" s="234"/>
       <c r="J46" s="55"/>
       <c r="K46" s="55"/>
       <c r="L46" s="2"/>
       <c r="M46" s="8"/>
     </row>
-    <row r="47" spans="1:13" ht="74" customHeight="1">
+    <row r="47" spans="1:13" ht="73.95" customHeight="1">
       <c r="A47" s="7"/>
       <c r="B47" s="56" t="s">
         <v>18</v>
@@ -4450,14 +4501,14 @@
       <c r="E47" s="57"/>
       <c r="F47" s="58"/>
       <c r="G47" s="58"/>
-      <c r="H47" s="212"/>
-      <c r="I47" s="212"/>
+      <c r="H47" s="229"/>
+      <c r="I47" s="230"/>
       <c r="J47" s="58"/>
       <c r="K47" s="58"/>
       <c r="L47" s="2"/>
       <c r="M47" s="8"/>
     </row>
-    <row r="48" spans="1:13" ht="74" customHeight="1">
+    <row r="48" spans="1:13" ht="73.95" customHeight="1">
       <c r="A48" s="7"/>
       <c r="B48" s="114"/>
       <c r="C48" s="115"/>
@@ -4472,7 +4523,7 @@
       <c r="L48" s="2"/>
       <c r="M48" s="8"/>
     </row>
-    <row r="49" spans="1:13" ht="74" customHeight="1">
+    <row r="49" spans="1:13" ht="73.95" customHeight="1">
       <c r="A49" s="7"/>
       <c r="B49" s="61" t="s">
         <v>50</v>
@@ -4486,16 +4537,16 @@
       <c r="G49" s="65" t="s">
         <v>51</v>
       </c>
-      <c r="H49" s="213" t="s">
+      <c r="H49" s="222" t="s">
         <v>54</v>
       </c>
-      <c r="I49" s="214"/>
+      <c r="I49" s="223"/>
       <c r="J49" s="65"/>
       <c r="K49" s="65"/>
       <c r="L49" s="2"/>
       <c r="M49" s="8"/>
     </row>
-    <row r="50" spans="1:13" ht="74" customHeight="1">
+    <row r="50" spans="1:13" ht="73.95" customHeight="1">
       <c r="A50" s="7"/>
       <c r="B50" s="118"/>
       <c r="C50" s="119"/>
@@ -4514,7 +4565,7 @@
       <c r="L50" s="2"/>
       <c r="M50" s="8"/>
     </row>
-    <row r="51" spans="1:13" ht="74" customHeight="1">
+    <row r="51" spans="1:13" ht="73.95" customHeight="1">
       <c r="A51" s="7"/>
       <c r="B51" s="61" t="s">
         <v>40</v>
@@ -4526,16 +4577,16 @@
       <c r="G51" s="65" t="s">
         <v>22</v>
       </c>
-      <c r="H51" s="213" t="s">
+      <c r="H51" s="184" t="s">
         <v>52</v>
       </c>
-      <c r="I51" s="214"/>
+      <c r="I51" s="185"/>
       <c r="J51" s="65"/>
       <c r="K51" s="65"/>
       <c r="L51" s="2"/>
       <c r="M51" s="8"/>
     </row>
-    <row r="52" spans="1:13" ht="74" customHeight="1">
+    <row r="52" spans="1:13" ht="73.95" customHeight="1">
       <c r="A52" s="7"/>
       <c r="B52" s="100"/>
       <c r="C52" s="101"/>
@@ -4550,7 +4601,7 @@
       <c r="L52" s="2"/>
       <c r="M52" s="8"/>
     </row>
-    <row r="53" spans="1:13" ht="74" customHeight="1">
+    <row r="53" spans="1:13" ht="73.95" customHeight="1">
       <c r="A53" s="7"/>
       <c r="B53" s="99" t="s">
         <v>49</v>
@@ -4564,16 +4615,16 @@
       <c r="G53" s="34" t="s">
         <v>32</v>
       </c>
-      <c r="H53" s="155" t="s">
+      <c r="H53" s="182" t="s">
         <v>38</v>
       </c>
-      <c r="I53" s="156"/>
+      <c r="I53" s="183"/>
       <c r="J53" s="30"/>
       <c r="K53" s="44"/>
       <c r="L53" s="2"/>
       <c r="M53" s="8"/>
     </row>
-    <row r="54" spans="1:13" ht="74" customHeight="1">
+    <row r="54" spans="1:13" ht="73.95" customHeight="1">
       <c r="A54" s="7"/>
       <c r="B54" s="68" t="s">
         <v>33</v>
@@ -4585,16 +4636,16 @@
       <c r="G54" s="44" t="s">
         <v>22</v>
       </c>
-      <c r="H54" s="210" t="s">
+      <c r="H54" s="181" t="s">
         <v>34</v>
       </c>
-      <c r="I54" s="210"/>
+      <c r="I54" s="181"/>
       <c r="J54" s="30"/>
       <c r="K54" s="30"/>
       <c r="L54" s="2"/>
       <c r="M54" s="8"/>
     </row>
-    <row r="55" spans="1:13" ht="74" customHeight="1">
+    <row r="55" spans="1:13" ht="73.95" customHeight="1">
       <c r="A55" s="7"/>
       <c r="B55" s="38"/>
       <c r="C55" s="39"/>
@@ -4602,14 +4653,14 @@
       <c r="E55" s="39"/>
       <c r="F55" s="40"/>
       <c r="G55" s="40"/>
-      <c r="H55" s="209"/>
-      <c r="I55" s="209"/>
+      <c r="H55" s="180"/>
+      <c r="I55" s="180"/>
       <c r="J55" s="45"/>
       <c r="K55" s="45"/>
       <c r="L55" s="2"/>
       <c r="M55" s="8"/>
     </row>
-    <row r="56" spans="1:13" ht="74" customHeight="1">
+    <row r="56" spans="1:13" ht="73.95" customHeight="1">
       <c r="A56" s="7"/>
       <c r="B56" s="46"/>
       <c r="C56" s="47"/>
@@ -4617,14 +4668,14 @@
       <c r="E56" s="47"/>
       <c r="F56" s="47"/>
       <c r="G56" s="47"/>
-      <c r="H56" s="224"/>
-      <c r="I56" s="225"/>
+      <c r="H56" s="176"/>
+      <c r="I56" s="177"/>
       <c r="J56" s="48"/>
       <c r="K56" s="47"/>
       <c r="L56" s="2"/>
       <c r="M56" s="8"/>
     </row>
-    <row r="57" spans="1:13" ht="74" customHeight="1">
+    <row r="57" spans="1:13" ht="73.95" customHeight="1">
       <c r="A57" s="7"/>
       <c r="B57" s="49"/>
       <c r="C57" s="50"/>
@@ -4632,14 +4683,14 @@
       <c r="E57" s="50"/>
       <c r="F57" s="50"/>
       <c r="G57" s="50"/>
-      <c r="H57" s="205"/>
-      <c r="I57" s="206"/>
+      <c r="H57" s="178"/>
+      <c r="I57" s="179"/>
       <c r="J57" s="51"/>
       <c r="K57" s="50"/>
       <c r="L57" s="2"/>
       <c r="M57" s="8"/>
     </row>
-    <row r="58" spans="1:13" ht="74" customHeight="1">
+    <row r="58" spans="1:13" ht="73.95" customHeight="1">
       <c r="A58" s="7"/>
       <c r="B58" s="12"/>
       <c r="C58" s="12"/>
@@ -4647,14 +4698,14 @@
       <c r="E58" s="12"/>
       <c r="F58" s="12"/>
       <c r="G58" s="12"/>
-      <c r="H58" s="217"/>
-      <c r="I58" s="217"/>
+      <c r="H58" s="170"/>
+      <c r="I58" s="170"/>
       <c r="J58" s="13"/>
       <c r="K58" s="12"/>
       <c r="L58" s="2"/>
       <c r="M58" s="8"/>
     </row>
-    <row r="59" spans="1:13" ht="74" customHeight="1">
+    <row r="59" spans="1:13" ht="73.95" customHeight="1">
       <c r="A59" s="7"/>
       <c r="B59" s="14"/>
       <c r="C59" s="15"/>
@@ -4662,14 +4713,14 @@
       <c r="E59" s="15"/>
       <c r="F59" s="15"/>
       <c r="G59" s="15"/>
-      <c r="H59" s="215"/>
-      <c r="I59" s="216"/>
+      <c r="H59" s="168"/>
+      <c r="I59" s="169"/>
       <c r="J59" s="16"/>
       <c r="K59" s="17"/>
       <c r="L59" s="2"/>
       <c r="M59" s="8"/>
     </row>
-    <row r="60" spans="1:13" ht="74" customHeight="1">
+    <row r="60" spans="1:13" ht="73.95" customHeight="1">
       <c r="A60" s="7"/>
       <c r="B60" s="18"/>
       <c r="C60" s="15"/>
@@ -4677,14 +4728,14 @@
       <c r="E60" s="15"/>
       <c r="F60" s="15"/>
       <c r="G60" s="15"/>
-      <c r="H60" s="215"/>
-      <c r="I60" s="216"/>
+      <c r="H60" s="168"/>
+      <c r="I60" s="169"/>
       <c r="J60" s="16"/>
       <c r="K60" s="17"/>
       <c r="L60" s="2"/>
       <c r="M60" s="8"/>
     </row>
-    <row r="61" spans="1:13" ht="74" customHeight="1">
+    <row r="61" spans="1:13" ht="73.95" customHeight="1">
       <c r="A61" s="7"/>
       <c r="B61" s="18"/>
       <c r="C61" s="15"/>
@@ -4692,14 +4743,14 @@
       <c r="E61" s="15"/>
       <c r="F61" s="15"/>
       <c r="G61" s="15"/>
-      <c r="H61" s="215"/>
-      <c r="I61" s="216"/>
+      <c r="H61" s="168"/>
+      <c r="I61" s="169"/>
       <c r="J61" s="16"/>
       <c r="K61" s="17"/>
       <c r="L61" s="2"/>
       <c r="M61" s="2"/>
     </row>
-    <row r="62" spans="1:13" ht="74" customHeight="1">
+    <row r="62" spans="1:13" ht="73.95" customHeight="1">
       <c r="A62" s="7"/>
       <c r="B62" s="18"/>
       <c r="C62" s="15"/>
@@ -4707,14 +4758,14 @@
       <c r="E62" s="15"/>
       <c r="F62" s="15"/>
       <c r="G62" s="15"/>
-      <c r="H62" s="215"/>
-      <c r="I62" s="216"/>
+      <c r="H62" s="168"/>
+      <c r="I62" s="169"/>
       <c r="J62" s="16"/>
       <c r="K62" s="17"/>
       <c r="L62" s="2"/>
       <c r="M62" s="2"/>
     </row>
-    <row r="63" spans="1:13" ht="16">
+    <row r="63" spans="1:13" ht="15.6">
       <c r="A63" s="2"/>
       <c r="B63" s="2"/>
       <c r="C63" s="2"/>
@@ -4729,7 +4780,7 @@
       <c r="L63" s="9"/>
       <c r="M63" s="10"/>
     </row>
-    <row r="64" spans="1:13" ht="16">
+    <row r="64" spans="1:13" ht="15.6">
       <c r="A64" s="2"/>
       <c r="B64" s="2"/>
       <c r="C64" s="2"/>
@@ -4854,11 +4905,59 @@
     </row>
   </sheetData>
   <mergeCells count="74">
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="C13:E13"/>
-    <mergeCell ref="C14:E14"/>
-    <mergeCell ref="F14:I15"/>
-    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="H33:I33"/>
+    <mergeCell ref="H34:I34"/>
+    <mergeCell ref="H22:I22"/>
+    <mergeCell ref="H42:I42"/>
+    <mergeCell ref="H25:I25"/>
+    <mergeCell ref="H27:I27"/>
+    <mergeCell ref="H26:I26"/>
+    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="H43:I43"/>
+    <mergeCell ref="H39:I39"/>
+    <mergeCell ref="H40:I40"/>
+    <mergeCell ref="H36:I36"/>
+    <mergeCell ref="H37:I37"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="C2:E2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="H2:K2"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="F3:G13"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="C6:E6"/>
+    <mergeCell ref="C7:E7"/>
+    <mergeCell ref="C8:E8"/>
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="C9:E9"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="C11:E11"/>
+    <mergeCell ref="H57:I57"/>
+    <mergeCell ref="H44:I44"/>
+    <mergeCell ref="H55:I55"/>
+    <mergeCell ref="H54:I54"/>
+    <mergeCell ref="H46:I46"/>
+    <mergeCell ref="H45:I45"/>
+    <mergeCell ref="H47:I47"/>
+    <mergeCell ref="H53:I53"/>
+    <mergeCell ref="H49:I49"/>
+    <mergeCell ref="H51:I51"/>
     <mergeCell ref="H61:I61"/>
     <mergeCell ref="H62:I62"/>
     <mergeCell ref="H58:I58"/>
@@ -4875,59 +4974,11 @@
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="H31:I31"/>
     <mergeCell ref="H24:I24"/>
-    <mergeCell ref="H57:I57"/>
-    <mergeCell ref="H44:I44"/>
-    <mergeCell ref="H55:I55"/>
-    <mergeCell ref="H54:I54"/>
-    <mergeCell ref="H46:I46"/>
-    <mergeCell ref="H45:I45"/>
-    <mergeCell ref="H47:I47"/>
-    <mergeCell ref="H53:I53"/>
-    <mergeCell ref="H49:I49"/>
-    <mergeCell ref="H51:I51"/>
-    <mergeCell ref="C2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="H2:K2"/>
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="F3:G13"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="C6:E6"/>
-    <mergeCell ref="C7:E7"/>
-    <mergeCell ref="C8:E8"/>
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="C9:E9"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="C11:E11"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="J10:K10"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="H43:I43"/>
-    <mergeCell ref="H39:I39"/>
-    <mergeCell ref="H40:I40"/>
-    <mergeCell ref="H36:I36"/>
-    <mergeCell ref="H37:I37"/>
-    <mergeCell ref="H18:I18"/>
-    <mergeCell ref="H33:I33"/>
-    <mergeCell ref="H34:I34"/>
-    <mergeCell ref="H22:I22"/>
-    <mergeCell ref="H42:I42"/>
-    <mergeCell ref="H25:I25"/>
-    <mergeCell ref="H27:I27"/>
-    <mergeCell ref="H26:I26"/>
-    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="F14:I15"/>
+    <mergeCell ref="H13:I13"/>
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
   <printOptions horizontalCentered="1"/>

</xml_diff>